<commit_message>
chore: atualizar planilha CONTAS-A-RECEBER
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/CONTAS-A-RECEBER.xlsx
+++ b/planilhas/CONTAS-A-RECEBER.xlsx
@@ -9,14 +9,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Relatório!$A$5:$S$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$78</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$82</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -40,7 +40,7 @@
     </r>
   </si>
   <si>
-    <t>Relatório exportado em quinta-feira, 21 de maio de 2026 por KAROL MEDEIROS</t>
+    <t>Relatório exportado em sexta-feira, 22 de maio de 2026 por KAROL MEDEIROS</t>
   </si>
   <si>
     <t>Conta de Recebimento</t>
@@ -235,132 +235,144 @@
     <t>YAGO ELIAS COSTA BATISTA</t>
   </si>
   <si>
+    <t>FA-11473</t>
+  </si>
+  <si>
+    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
+  </si>
+  <si>
+    <t>FA-11478</t>
+  </si>
+  <si>
+    <t>FA-11614</t>
+  </si>
+  <si>
+    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11453</t>
+  </si>
+  <si>
+    <t>FA-11390</t>
+  </si>
+  <si>
+    <t>FA-11458</t>
+  </si>
+  <si>
+    <t>FA-11615</t>
+  </si>
+  <si>
+    <t>FA-11396</t>
+  </si>
+  <si>
+    <t>FA-11525</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11559</t>
+  </si>
+  <si>
+    <t>FA-11497</t>
+  </si>
+  <si>
+    <t>ANDRE CAVALCANTI DA FE</t>
+  </si>
+  <si>
+    <t>FA-11466</t>
+  </si>
+  <si>
+    <t>FA-11474</t>
+  </si>
+  <si>
+    <t>FA-11560</t>
+  </si>
+  <si>
+    <t>DIEGO TAYAO DANTAS</t>
+  </si>
+  <si>
+    <t>FA-11481</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11402</t>
+  </si>
+  <si>
+    <t>FA-11616</t>
+  </si>
+  <si>
+    <t>FA-11620</t>
+  </si>
+  <si>
+    <t>FA-11482</t>
+  </si>
+  <si>
+    <t>FA-11483</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11484</t>
+  </si>
+  <si>
+    <t>FA-11561</t>
+  </si>
+  <si>
+    <t>ELSON VIEIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11675</t>
+  </si>
+  <si>
+    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
+  </si>
+  <si>
+    <t>FA-11479</t>
+  </si>
+  <si>
+    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11461</t>
+  </si>
+  <si>
+    <t>FA-11279</t>
+  </si>
+  <si>
+    <t>FELIPE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11476</t>
+  </si>
+  <si>
+    <t>FA-11674</t>
+  </si>
+  <si>
+    <t>FA-11611</t>
+  </si>
+  <si>
+    <t>M&amp;S DO TRABALHO</t>
+  </si>
+  <si>
+    <t>FA-11496</t>
+  </si>
+  <si>
+    <t>FA-11464</t>
+  </si>
+  <si>
+    <t>FA-11667</t>
+  </si>
+  <si>
+    <t>HOJE</t>
+  </si>
+  <si>
     <t>FA-11399</t>
   </si>
   <si>
-    <t>FA-11473</t>
-  </si>
-  <si>
-    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
-  </si>
-  <si>
-    <t>FA-11478</t>
-  </si>
-  <si>
-    <t>FA-11496</t>
-  </si>
-  <si>
-    <t>ANDRE CAVALCANTI DA FE</t>
-  </si>
-  <si>
-    <t>FA-11614</t>
-  </si>
-  <si>
-    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11453</t>
-  </si>
-  <si>
-    <t>FA-11390</t>
-  </si>
-  <si>
-    <t>FA-11458</t>
-  </si>
-  <si>
-    <t>FA-11615</t>
-  </si>
-  <si>
-    <t>FA-11396</t>
-  </si>
-  <si>
-    <t>FA-11525</t>
-  </si>
-  <si>
-    <t>ROBERTO MURATORI</t>
-  </si>
-  <si>
-    <t>FA-11559</t>
-  </si>
-  <si>
-    <t>FA-11497</t>
-  </si>
-  <si>
-    <t>FA-11466</t>
-  </si>
-  <si>
-    <t>FA-11474</t>
-  </si>
-  <si>
-    <t>FA-11560</t>
-  </si>
-  <si>
-    <t>DIEGO TAYAO DANTAS</t>
-  </si>
-  <si>
-    <t>FA-11481</t>
-  </si>
-  <si>
-    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
-  </si>
-  <si>
-    <t>FA-11402</t>
-  </si>
-  <si>
-    <t>FA-11616</t>
-  </si>
-  <si>
-    <t>FA-11620</t>
-  </si>
-  <si>
-    <t>FA-11482</t>
-  </si>
-  <si>
-    <t>FA-11483</t>
-  </si>
-  <si>
-    <t>LUCAS NAJA MOURA RODRIGUES</t>
-  </si>
-  <si>
-    <t>FA-11484</t>
-  </si>
-  <si>
-    <t>FA-11561</t>
-  </si>
-  <si>
-    <t>ELSON VIEIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11479</t>
-  </si>
-  <si>
-    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11461</t>
-  </si>
-  <si>
-    <t>FA-11279</t>
-  </si>
-  <si>
-    <t>FELIPE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11476</t>
-  </si>
-  <si>
-    <t>FA-11611</t>
-  </si>
-  <si>
-    <t>M&amp;S DO TRABALHO</t>
-  </si>
-  <si>
-    <t>FA-11464</t>
-  </si>
-  <si>
-    <t>FA-11667</t>
-  </si>
-  <si>
     <t>A VENCER</t>
   </si>
   <si>
@@ -388,6 +400,12 @@
     <t>FA-11668</t>
   </si>
   <si>
+    <t>FA-11683</t>
+  </si>
+  <si>
+    <t>GILVAN RODRIGUES MACHADO</t>
+  </si>
+  <si>
     <t>FA-11656</t>
   </si>
   <si>
@@ -427,25 +445,28 @@
     <t>FA-11564</t>
   </si>
   <si>
+    <t>FA-11676</t>
+  </si>
+  <si>
     <t>FA-11329</t>
   </si>
   <si>
     <t>MAICON LOPES SILVA</t>
   </si>
   <si>
+    <t>FA-11632</t>
+  </si>
+  <si>
+    <t>TANIELLE GLAUCIANA SOUZA DA SILVA</t>
+  </si>
+  <si>
+    <t>PÚBLICO</t>
+  </si>
+  <si>
     <t>FA-11644</t>
   </si>
   <si>
     <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
-  </si>
-  <si>
-    <t>PÚBLICO</t>
-  </si>
-  <si>
-    <t>FA-11632</t>
-  </si>
-  <si>
-    <t>TANIELLE GLAUCIANA SOUZA DA SILVA</t>
   </si>
   <si>
     <t>FA-11613</t>
@@ -597,7 +618,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName=""/>
-  <dimension ref="A1:S84"/>
+  <dimension ref="A1:S88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38.13657760620117" customWidth="1" style="1"/>
@@ -714,10 +735,10 @@
         <v>23</v>
       </c>
       <c r="F6" s="8">
-        <v>-45</v>
+        <v>-46</v>
       </c>
       <c r="G6" s="8">
-        <v>-31</v>
+        <v>-32</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>24</v>
@@ -773,10 +794,10 @@
         <v>23</v>
       </c>
       <c r="F7" s="8">
-        <v>-38</v>
+        <v>-39</v>
       </c>
       <c r="G7" s="8">
-        <v>-29</v>
+        <v>-30</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>24</v>
@@ -832,10 +853,10 @@
         <v>23</v>
       </c>
       <c r="F8" s="8">
-        <v>-38</v>
+        <v>-39</v>
       </c>
       <c r="G8" s="8">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>24</v>
@@ -891,10 +912,10 @@
         <v>46127</v>
       </c>
       <c r="F9" s="8">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="G9" s="8">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>30</v>
@@ -950,10 +971,10 @@
         <v>46097</v>
       </c>
       <c r="F10" s="8">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="G10" s="8">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>30</v>
@@ -1009,10 +1030,10 @@
         <v>23</v>
       </c>
       <c r="F11" s="8">
-        <v>-31</v>
+        <v>-32</v>
       </c>
       <c r="G11" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>24</v>
@@ -1068,10 +1089,10 @@
         <v>23</v>
       </c>
       <c r="F12" s="8">
-        <v>-38</v>
+        <v>-39</v>
       </c>
       <c r="G12" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>24</v>
@@ -1127,10 +1148,10 @@
         <v>46141</v>
       </c>
       <c r="F13" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="G13" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>30</v>
@@ -1186,10 +1207,10 @@
         <v>23</v>
       </c>
       <c r="F14" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G14" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>30</v>
@@ -1245,10 +1266,10 @@
         <v>23</v>
       </c>
       <c r="F15" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G15" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>30</v>
@@ -1304,10 +1325,10 @@
         <v>46097</v>
       </c>
       <c r="F16" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G16" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>30</v>
@@ -1363,10 +1384,10 @@
         <v>23</v>
       </c>
       <c r="F17" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G17" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>30</v>
@@ -1422,10 +1443,10 @@
         <v>46141</v>
       </c>
       <c r="F18" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G18" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>30</v>
@@ -1481,10 +1502,10 @@
         <v>23</v>
       </c>
       <c r="F19" s="8">
-        <v>-31</v>
+        <v>-32</v>
       </c>
       <c r="G19" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>24</v>
@@ -1540,10 +1561,10 @@
         <v>23</v>
       </c>
       <c r="F20" s="8">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="G20" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>30</v>
@@ -1599,10 +1620,10 @@
         <v>46148</v>
       </c>
       <c r="F21" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G21" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>30</v>
@@ -1658,10 +1679,10 @@
         <v>23</v>
       </c>
       <c r="F22" s="8">
-        <v>-38</v>
+        <v>-39</v>
       </c>
       <c r="G22" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>24</v>
@@ -1717,10 +1738,10 @@
         <v>23</v>
       </c>
       <c r="F23" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G23" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>30</v>
@@ -1776,10 +1797,10 @@
         <v>46153</v>
       </c>
       <c r="F24" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="G24" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>30</v>
@@ -1835,10 +1856,10 @@
         <v>23</v>
       </c>
       <c r="F25" s="8">
-        <v>-225</v>
+        <v>-226</v>
       </c>
       <c r="G25" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>62</v>
@@ -1894,10 +1915,10 @@
         <v>46097</v>
       </c>
       <c r="F26" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G26" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>30</v>
@@ -1953,10 +1974,10 @@
         <v>46141</v>
       </c>
       <c r="F27" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G27" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>30</v>
@@ -2012,10 +2033,10 @@
         <v>46119</v>
       </c>
       <c r="F28" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G28" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>30</v>
@@ -2068,13 +2089,13 @@
         <v>46153</v>
       </c>
       <c r="E29" s="7">
-        <v>46112</v>
+        <v>46119</v>
       </c>
       <c r="F29" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G29" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>30</v>
@@ -2089,10 +2110,10 @@
         <v>23</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="N29" s="6" t="s">
         <v>27</v>
@@ -2110,7 +2131,7 @@
         <v>29</v>
       </c>
       <c r="S29" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="30" ht="23" customHeight="1">
@@ -2130,10 +2151,10 @@
         <v>46119</v>
       </c>
       <c r="F30" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G30" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>30</v>
@@ -2142,16 +2163,16 @@
         <v>30</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K30" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="N30" s="6" t="s">
         <v>27</v>
@@ -2166,10 +2187,10 @@
         <v>37</v>
       </c>
       <c r="R30" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S30" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="31" ht="23" customHeight="1">
@@ -2177,19 +2198,19 @@
         <v>22</v>
       </c>
       <c r="B31" s="7">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="C31" s="7">
-        <v>46153</v>
+        <v>46146</v>
       </c>
       <c r="D31" s="7">
-        <v>46153</v>
-      </c>
-      <c r="E31" s="7">
-        <v>46119</v>
+        <v>46146</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F31" s="8">
-        <v>-10</v>
+        <v>-18</v>
       </c>
       <c r="G31" s="8">
         <v>-10</v>
@@ -2207,7 +2228,7 @@
         <v>23</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="M31" s="6" t="s">
         <v>23</v>
@@ -2222,13 +2243,13 @@
         <v>23</v>
       </c>
       <c r="Q31" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S31" s="9">
-        <v>680</v>
+        <v>280</v>
       </c>
     </row>
     <row r="32" ht="23" customHeight="1">
@@ -2239,19 +2260,19 @@
         <v>46154</v>
       </c>
       <c r="C32" s="7">
-        <v>46125</v>
+        <v>46132</v>
       </c>
       <c r="D32" s="7">
-        <v>46125</v>
+        <v>46132</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F32" s="8">
-        <v>-38</v>
+        <v>-32</v>
       </c>
       <c r="G32" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>24</v>
@@ -2260,16 +2281,16 @@
         <v>30</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="N32" s="6" t="s">
         <v>27</v>
@@ -2284,10 +2305,10 @@
         <v>23</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S32" s="9">
-        <v>150</v>
+        <v>317.54</v>
       </c>
     </row>
     <row r="33" ht="23" customHeight="1">
@@ -2295,25 +2316,25 @@
         <v>22</v>
       </c>
       <c r="B33" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="C33" s="7">
-        <v>46146</v>
+        <v>46132</v>
       </c>
       <c r="D33" s="7">
-        <v>46146</v>
+        <v>46132</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F33" s="8">
-        <v>-17</v>
+        <v>-32</v>
       </c>
       <c r="G33" s="8">
         <v>-9</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="I33" s="6" t="s">
         <v>30</v>
@@ -2325,7 +2346,7 @@
         <v>23</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="M33" s="6" t="s">
         <v>23</v>
@@ -2346,7 +2367,7 @@
         <v>29</v>
       </c>
       <c r="S33" s="9">
-        <v>280</v>
+        <v>140</v>
       </c>
     </row>
     <row r="34" ht="23" customHeight="1">
@@ -2354,40 +2375,40 @@
         <v>22</v>
       </c>
       <c r="B34" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="C34" s="7">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="D34" s="7">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F34" s="8">
-        <v>-31</v>
+        <v>-25</v>
       </c>
       <c r="G34" s="8">
         <v>-9</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>30</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K34" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>27</v>
@@ -2405,7 +2426,7 @@
         <v>29</v>
       </c>
       <c r="S34" s="9">
-        <v>317.54</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" ht="23" customHeight="1">
@@ -2416,34 +2437,34 @@
         <v>46155</v>
       </c>
       <c r="C35" s="7">
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="D35" s="7">
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F35" s="8">
-        <v>-31</v>
+        <v>-11</v>
       </c>
       <c r="G35" s="8">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>30</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>23</v>
@@ -2464,7 +2485,7 @@
         <v>29</v>
       </c>
       <c r="S35" s="9">
-        <v>140</v>
+        <v>530</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1">
@@ -2472,19 +2493,19 @@
         <v>22</v>
       </c>
       <c r="B36" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="C36" s="7">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="D36" s="7">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F36" s="8">
-        <v>-24</v>
+        <v>-18</v>
       </c>
       <c r="G36" s="8">
         <v>-8</v>
@@ -2496,16 +2517,16 @@
         <v>30</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="N36" s="6" t="s">
         <v>27</v>
@@ -2523,7 +2544,7 @@
         <v>29</v>
       </c>
       <c r="S36" s="9">
-        <v>250</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" ht="23" customHeight="1">
@@ -2531,22 +2552,22 @@
         <v>22</v>
       </c>
       <c r="B37" s="7">
-        <v>46155</v>
+        <v>46160</v>
       </c>
       <c r="C37" s="7">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="D37" s="7">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F37" s="8">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="G37" s="8">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>30</v>
@@ -2555,13 +2576,13 @@
         <v>30</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>23</v>
@@ -2582,7 +2603,7 @@
         <v>29</v>
       </c>
       <c r="S37" s="9">
-        <v>530</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="38" ht="23" customHeight="1">
@@ -2590,22 +2611,22 @@
         <v>22</v>
       </c>
       <c r="B38" s="7">
-        <v>46156</v>
+        <v>46160</v>
       </c>
       <c r="C38" s="7">
-        <v>46146</v>
+        <v>46082</v>
       </c>
       <c r="D38" s="7">
-        <v>46146</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>23</v>
+        <v>46160</v>
+      </c>
+      <c r="E38" s="7">
+        <v>46097</v>
       </c>
       <c r="F38" s="8">
-        <v>-17</v>
+        <v>-4</v>
       </c>
       <c r="G38" s="8">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>30</v>
@@ -2614,13 +2635,13 @@
         <v>30</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>23</v>
@@ -2635,13 +2656,13 @@
         <v>23</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="R38" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S38" s="9">
-        <v>130</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="39" ht="23" customHeight="1">
@@ -2657,14 +2678,14 @@
       <c r="D39" s="7">
         <v>46160</v>
       </c>
-      <c r="E39" s="7" t="s">
-        <v>23</v>
+      <c r="E39" s="7">
+        <v>46127</v>
       </c>
       <c r="F39" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G39" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>30</v>
@@ -2673,16 +2694,16 @@
         <v>30</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="K39" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="N39" s="6" t="s">
         <v>27</v>
@@ -2694,13 +2715,13 @@
         <v>23</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R39" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S39" s="9">
-        <v>97.5</v>
+        <v>172</v>
       </c>
     </row>
     <row r="40" ht="23" customHeight="1">
@@ -2711,19 +2732,19 @@
         <v>46160</v>
       </c>
       <c r="C40" s="7">
-        <v>46082</v>
+        <v>46160</v>
       </c>
       <c r="D40" s="7">
         <v>46160</v>
       </c>
       <c r="E40" s="7">
-        <v>46097</v>
+        <v>46141</v>
       </c>
       <c r="F40" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G40" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H40" s="6" t="s">
         <v>30</v>
@@ -2732,13 +2753,13 @@
         <v>30</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>23</v>
@@ -2753,13 +2774,13 @@
         <v>23</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R40" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S40" s="9">
-        <v>146.55</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41" ht="23" customHeight="1">
@@ -2770,22 +2791,22 @@
         <v>46160</v>
       </c>
       <c r="C41" s="7">
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="D41" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E41" s="7">
-        <v>46127</v>
+        <v>46132</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F41" s="8">
-        <v>-3</v>
+        <v>-32</v>
       </c>
       <c r="G41" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="I41" s="6" t="s">
         <v>30</v>
@@ -2800,7 +2821,7 @@
         <v>81</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>81</v>
+        <v>23</v>
       </c>
       <c r="N41" s="6" t="s">
         <v>27</v>
@@ -2812,13 +2833,13 @@
         <v>23</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R41" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S41" s="9">
-        <v>172</v>
+        <v>350</v>
       </c>
     </row>
     <row r="42" ht="23" customHeight="1">
@@ -2829,19 +2850,19 @@
         <v>46160</v>
       </c>
       <c r="C42" s="7">
-        <v>46160</v>
+        <v>46146</v>
       </c>
       <c r="D42" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E42" s="7">
-        <v>46141</v>
+        <v>46146</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F42" s="8">
-        <v>-3</v>
+        <v>-18</v>
       </c>
       <c r="G42" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>30</v>
@@ -2856,10 +2877,10 @@
         <v>23</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="N42" s="6" t="s">
         <v>27</v>
@@ -2871,13 +2892,13 @@
         <v>23</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R42" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S42" s="9">
-        <v>310</v>
+        <v>450</v>
       </c>
     </row>
     <row r="43" ht="23" customHeight="1">
@@ -2888,22 +2909,22 @@
         <v>46160</v>
       </c>
       <c r="C43" s="7">
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="D43" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>23</v>
+        <v>46160</v>
+      </c>
+      <c r="E43" s="7">
+        <v>46119</v>
       </c>
       <c r="F43" s="8">
-        <v>-31</v>
+        <v>-4</v>
       </c>
       <c r="G43" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I43" s="6" t="s">
         <v>30</v>
@@ -2915,10 +2936,10 @@
         <v>23</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="N43" s="6" t="s">
         <v>27</v>
@@ -2930,13 +2951,13 @@
         <v>23</v>
       </c>
       <c r="Q43" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R43" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S43" s="9">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="44" ht="23" customHeight="1">
@@ -2947,19 +2968,19 @@
         <v>46160</v>
       </c>
       <c r="C44" s="7">
-        <v>46146</v>
+        <v>46160</v>
       </c>
       <c r="D44" s="7">
-        <v>46146</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>23</v>
+        <v>46160</v>
+      </c>
+      <c r="E44" s="7">
+        <v>46141</v>
       </c>
       <c r="F44" s="8">
-        <v>-17</v>
+        <v>-4</v>
       </c>
       <c r="G44" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>30</v>
@@ -2974,10 +2995,10 @@
         <v>23</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="N44" s="6" t="s">
         <v>27</v>
@@ -2989,13 +3010,13 @@
         <v>23</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R44" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S44" s="9">
-        <v>450</v>
+        <v>620</v>
       </c>
     </row>
     <row r="45" ht="23" customHeight="1">
@@ -3015,10 +3036,10 @@
         <v>46119</v>
       </c>
       <c r="F45" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G45" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>30</v>
@@ -3027,16 +3048,16 @@
         <v>30</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="N45" s="6" t="s">
         <v>27</v>
@@ -3051,10 +3072,10 @@
         <v>37</v>
       </c>
       <c r="R45" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S45" s="9">
-        <v>600</v>
+        <v>620</v>
       </c>
     </row>
     <row r="46" ht="23" customHeight="1">
@@ -3071,13 +3092,13 @@
         <v>46160</v>
       </c>
       <c r="E46" s="7">
-        <v>46141</v>
+        <v>46112</v>
       </c>
       <c r="F46" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G46" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>30</v>
@@ -3086,16 +3107,16 @@
         <v>30</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="N46" s="6" t="s">
         <v>27</v>
@@ -3113,7 +3134,7 @@
         <v>29</v>
       </c>
       <c r="S46" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="47" ht="23" customHeight="1">
@@ -3130,13 +3151,13 @@
         <v>46160</v>
       </c>
       <c r="E47" s="7">
-        <v>46119</v>
+        <v>46150</v>
       </c>
       <c r="F47" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G47" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>30</v>
@@ -3145,16 +3166,16 @@
         <v>30</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K47" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="M47" s="6" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="N47" s="6" t="s">
         <v>27</v>
@@ -3169,10 +3190,10 @@
         <v>37</v>
       </c>
       <c r="R47" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S47" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="48" ht="23" customHeight="1">
@@ -3189,13 +3210,13 @@
         <v>46160</v>
       </c>
       <c r="E48" s="7">
-        <v>46112</v>
+        <v>46153</v>
       </c>
       <c r="F48" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G48" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>30</v>
@@ -3210,7 +3231,7 @@
         <v>23</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="M48" s="6" t="s">
         <v>23</v>
@@ -3231,7 +3252,7 @@
         <v>29</v>
       </c>
       <c r="S48" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="49" ht="23" customHeight="1">
@@ -3248,13 +3269,13 @@
         <v>46160</v>
       </c>
       <c r="E49" s="7">
-        <v>46150</v>
+        <v>46119</v>
       </c>
       <c r="F49" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G49" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>30</v>
@@ -3269,10 +3290,10 @@
         <v>23</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="N49" s="6" t="s">
         <v>27</v>
@@ -3290,7 +3311,7 @@
         <v>29</v>
       </c>
       <c r="S49" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="50" ht="23" customHeight="1">
@@ -3307,13 +3328,13 @@
         <v>46160</v>
       </c>
       <c r="E50" s="7">
-        <v>46153</v>
+        <v>46119</v>
       </c>
       <c r="F50" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H50" s="6" t="s">
         <v>30</v>
@@ -3328,7 +3349,7 @@
         <v>23</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>23</v>
@@ -3349,7 +3370,7 @@
         <v>29</v>
       </c>
       <c r="S50" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="51" ht="23" customHeight="1">
@@ -3369,10 +3390,10 @@
         <v>46119</v>
       </c>
       <c r="F51" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G51" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>30</v>
@@ -3381,16 +3402,16 @@
         <v>30</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K51" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="N51" s="6" t="s">
         <v>27</v>
@@ -3405,10 +3426,10 @@
         <v>37</v>
       </c>
       <c r="R51" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S51" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="52" ht="23" customHeight="1">
@@ -3425,13 +3446,13 @@
         <v>46160</v>
       </c>
       <c r="E52" s="7">
-        <v>46119</v>
+        <v>46141</v>
       </c>
       <c r="F52" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G52" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>30</v>
@@ -3440,13 +3461,13 @@
         <v>30</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K52" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M52" s="6" t="s">
         <v>23</v>
@@ -3464,7 +3485,7 @@
         <v>37</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S52" s="9">
         <v>680</v>
@@ -3484,13 +3505,13 @@
         <v>46160</v>
       </c>
       <c r="E53" s="7">
-        <v>46119</v>
+        <v>46164</v>
       </c>
       <c r="F53" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G53" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>30</v>
@@ -3499,13 +3520,13 @@
         <v>30</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K53" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>32</v>
+        <v>98</v>
       </c>
       <c r="M53" s="6" t="s">
         <v>23</v>
@@ -3543,13 +3564,13 @@
         <v>46160</v>
       </c>
       <c r="E54" s="7">
-        <v>46141</v>
+        <v>46119</v>
       </c>
       <c r="F54" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G54" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>30</v>
@@ -3558,13 +3579,13 @@
         <v>30</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>23</v>
@@ -3576,16 +3597,16 @@
         <v>27</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>37</v>
       </c>
       <c r="R54" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S54" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="55" ht="23" customHeight="1">
@@ -3593,19 +3614,19 @@
         <v>22</v>
       </c>
       <c r="B55" s="7">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="C55" s="7">
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="D55" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E55" s="7">
-        <v>46119</v>
+        <v>46139</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F55" s="8">
-        <v>-3</v>
+        <v>-25</v>
       </c>
       <c r="G55" s="8">
         <v>-3</v>
@@ -3617,7 +3638,7 @@
         <v>30</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K55" s="6" t="s">
         <v>23</v>
@@ -3638,13 +3659,13 @@
         <v>28</v>
       </c>
       <c r="Q55" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R55" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S55" s="9">
-        <v>700</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" ht="23" customHeight="1">
@@ -3655,19 +3676,19 @@
         <v>46161</v>
       </c>
       <c r="C56" s="7">
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="D56" s="7">
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F56" s="8">
-        <v>-24</v>
+        <v>-4</v>
       </c>
       <c r="G56" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>30</v>
@@ -3676,13 +3697,13 @@
         <v>30</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>23</v>
@@ -3694,7 +3715,7 @@
         <v>27</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="Q56" s="6" t="s">
         <v>23</v>
@@ -3703,7 +3724,7 @@
         <v>29</v>
       </c>
       <c r="S56" s="9">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="57" ht="23" customHeight="1">
@@ -3714,20 +3735,20 @@
         <v>46161</v>
       </c>
       <c r="C57" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="D57" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F57" s="8">
+        <v>-11</v>
+      </c>
+      <c r="G57" s="8">
         <v>-3</v>
       </c>
-      <c r="G57" s="8">
-        <v>-2</v>
-      </c>
       <c r="H57" s="6" t="s">
         <v>30</v>
       </c>
@@ -3735,16 +3756,16 @@
         <v>30</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="N57" s="6" t="s">
         <v>27</v>
@@ -3759,10 +3780,10 @@
         <v>23</v>
       </c>
       <c r="R57" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S57" s="9">
-        <v>130</v>
+        <v>277.36</v>
       </c>
     </row>
     <row r="58" ht="23" customHeight="1">
@@ -3782,10 +3803,10 @@
         <v>23</v>
       </c>
       <c r="F58" s="8">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G58" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>30</v>
@@ -3794,16 +3815,16 @@
         <v>30</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K58" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="N58" s="6" t="s">
         <v>27</v>
@@ -3821,7 +3842,7 @@
         <v>33</v>
       </c>
       <c r="S58" s="9">
-        <v>277.36</v>
+        <v>280</v>
       </c>
     </row>
     <row r="59" ht="23" customHeight="1">
@@ -3841,10 +3862,10 @@
         <v>46149</v>
       </c>
       <c r="F59" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="G59" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H59" s="6" t="s">
         <v>30</v>
@@ -3853,16 +3874,16 @@
         <v>30</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K59" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M59" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N59" s="6" t="s">
         <v>27</v>
@@ -3891,37 +3912,37 @@
         <v>46162</v>
       </c>
       <c r="C60" s="7">
-        <v>46146</v>
+        <v>46125</v>
       </c>
       <c r="D60" s="7">
-        <v>46146</v>
+        <v>46125</v>
       </c>
       <c r="E60" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F60" s="8">
-        <v>-17</v>
+        <v>-39</v>
       </c>
       <c r="G60" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="I60" s="6" t="s">
         <v>30</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K60" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="N60" s="6" t="s">
         <v>27</v>
@@ -3936,10 +3957,10 @@
         <v>23</v>
       </c>
       <c r="R60" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S60" s="9">
-        <v>200</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61" ht="23" customHeight="1">
@@ -3947,46 +3968,46 @@
         <v>22</v>
       </c>
       <c r="B61" s="7">
-        <v>46164</v>
+        <v>46162</v>
       </c>
       <c r="C61" s="7">
-        <v>46160</v>
+        <v>46146</v>
       </c>
       <c r="D61" s="7">
-        <v>46160</v>
+        <v>46146</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F61" s="8">
-        <v>-3</v>
+        <v>-18</v>
       </c>
       <c r="G61" s="8">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="H61" s="6" t="s">
         <v>30</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K61" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="N61" s="6" t="s">
         <v>27</v>
       </c>
       <c r="O61" s="6" t="s">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="P61" s="6" t="s">
         <v>23</v>
@@ -3998,7 +4019,7 @@
         <v>29</v>
       </c>
       <c r="S61" s="9">
-        <v>290</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62" ht="23" customHeight="1">
@@ -4006,58 +4027,58 @@
         <v>22</v>
       </c>
       <c r="B62" s="7">
-        <v>46167</v>
+        <v>46164</v>
       </c>
       <c r="C62" s="7">
-        <v>46082</v>
+        <v>46160</v>
       </c>
       <c r="D62" s="7">
-        <v>46167</v>
-      </c>
-      <c r="E62" s="7">
-        <v>46097</v>
+        <v>46160</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F62" s="8">
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="G62" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="K62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="M62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="Q62" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="R62" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S62" s="9">
-        <v>146.55</v>
+        <v>290</v>
       </c>
     </row>
     <row r="63" ht="23" customHeight="1">
@@ -4068,55 +4089,55 @@
         <v>46167</v>
       </c>
       <c r="C63" s="7">
-        <v>46167</v>
+        <v>46153</v>
       </c>
       <c r="D63" s="7">
-        <v>46167</v>
-      </c>
-      <c r="E63" s="7">
-        <v>46119</v>
+        <v>46153</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F63" s="8">
-        <v>4</v>
+        <v>-11</v>
       </c>
       <c r="G63" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="M63" s="6" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="O63" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="Q63" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R63" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S63" s="9">
-        <v>600</v>
+        <v>130</v>
       </c>
     </row>
     <row r="64" ht="23" customHeight="1">
@@ -4127,19 +4148,19 @@
         <v>46167</v>
       </c>
       <c r="C64" s="7">
-        <v>46167</v>
+        <v>46082</v>
       </c>
       <c r="D64" s="7">
         <v>46167</v>
       </c>
       <c r="E64" s="7">
-        <v>46141</v>
+        <v>46097</v>
       </c>
       <c r="F64" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G64" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>23</v>
@@ -4148,34 +4169,34 @@
         <v>23</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>111</v>
+        <v>31</v>
       </c>
       <c r="K64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="M64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="Q64" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R64" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S64" s="9">
-        <v>620</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="65" ht="23" customHeight="1">
@@ -4192,13 +4213,13 @@
         <v>46167</v>
       </c>
       <c r="E65" s="7">
-        <v>46141</v>
+        <v>46119</v>
       </c>
       <c r="F65" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G65" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>23</v>
@@ -4207,22 +4228,22 @@
         <v>23</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K65" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O65" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P65" s="6" t="s">
         <v>23</v>
@@ -4234,7 +4255,7 @@
         <v>29</v>
       </c>
       <c r="S65" s="9">
-        <v>620</v>
+        <v>600</v>
       </c>
     </row>
     <row r="66" ht="23" customHeight="1">
@@ -4251,13 +4272,13 @@
         <v>46167</v>
       </c>
       <c r="E66" s="7">
-        <v>46119</v>
+        <v>46141</v>
       </c>
       <c r="F66" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G66" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>23</v>
@@ -4266,22 +4287,22 @@
         <v>23</v>
       </c>
       <c r="J66" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N66" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="K66" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>109</v>
-      </c>
       <c r="O66" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>23</v>
@@ -4290,7 +4311,7 @@
         <v>37</v>
       </c>
       <c r="R66" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S66" s="9">
         <v>620</v>
@@ -4310,13 +4331,13 @@
         <v>46167</v>
       </c>
       <c r="E67" s="7">
-        <v>46119</v>
+        <v>46141</v>
       </c>
       <c r="F67" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G67" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>23</v>
@@ -4325,25 +4346,25 @@
         <v>23</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K67" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="M67" s="6" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P67" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="Q67" s="6" t="s">
         <v>37</v>
@@ -4352,7 +4373,7 @@
         <v>29</v>
       </c>
       <c r="S67" s="9">
-        <v>630</v>
+        <v>620</v>
       </c>
     </row>
     <row r="68" ht="23" customHeight="1">
@@ -4369,13 +4390,13 @@
         <v>46167</v>
       </c>
       <c r="E68" s="7">
-        <v>46150</v>
+        <v>46119</v>
       </c>
       <c r="F68" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G68" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>23</v>
@@ -4384,22 +4405,22 @@
         <v>23</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K68" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="M68" s="6" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>23</v>
@@ -4408,10 +4429,10 @@
         <v>37</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S68" s="9">
-        <v>630</v>
+        <v>620</v>
       </c>
     </row>
     <row r="69" ht="23" customHeight="1">
@@ -4428,13 +4449,13 @@
         <v>46167</v>
       </c>
       <c r="E69" s="7">
-        <v>46163</v>
+        <v>46119</v>
       </c>
       <c r="F69" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G69" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H69" s="6" t="s">
         <v>23</v>
@@ -4443,25 +4464,25 @@
         <v>23</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K69" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O69" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P69" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="Q69" s="6" t="s">
         <v>37</v>
@@ -4487,13 +4508,13 @@
         <v>46167</v>
       </c>
       <c r="E70" s="7">
-        <v>46160</v>
+        <v>46150</v>
       </c>
       <c r="F70" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G70" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>23</v>
@@ -4502,22 +4523,22 @@
         <v>23</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K70" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>119</v>
+        <v>71</v>
       </c>
       <c r="M70" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>23</v>
@@ -4529,7 +4550,7 @@
         <v>29</v>
       </c>
       <c r="S70" s="9">
-        <v>650</v>
+        <v>630</v>
       </c>
     </row>
     <row r="71" ht="23" customHeight="1">
@@ -4546,13 +4567,13 @@
         <v>46167</v>
       </c>
       <c r="E71" s="7">
-        <v>46153</v>
+        <v>46163</v>
       </c>
       <c r="F71" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G71" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>23</v>
@@ -4561,22 +4582,22 @@
         <v>23</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K71" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M71" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O71" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P71" s="6" t="s">
         <v>23</v>
@@ -4588,7 +4609,7 @@
         <v>29</v>
       </c>
       <c r="S71" s="9">
-        <v>650</v>
+        <v>630</v>
       </c>
     </row>
     <row r="72" ht="23" customHeight="1">
@@ -4605,13 +4626,13 @@
         <v>46167</v>
       </c>
       <c r="E72" s="7">
-        <v>46127</v>
+        <v>46164</v>
       </c>
       <c r="F72" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G72" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>23</v>
@@ -4620,22 +4641,22 @@
         <v>23</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>23</v>
@@ -4647,7 +4668,7 @@
         <v>29</v>
       </c>
       <c r="S72" s="9">
-        <v>650</v>
+        <v>630</v>
       </c>
     </row>
     <row r="73" ht="23" customHeight="1">
@@ -4664,13 +4685,13 @@
         <v>46167</v>
       </c>
       <c r="E73" s="7">
-        <v>46119</v>
+        <v>46160</v>
       </c>
       <c r="F73" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G73" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H73" s="6" t="s">
         <v>23</v>
@@ -4679,22 +4700,22 @@
         <v>23</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="M73" s="6" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O73" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P73" s="6" t="s">
         <v>23</v>
@@ -4723,13 +4744,13 @@
         <v>46167</v>
       </c>
       <c r="E74" s="7">
-        <v>46092</v>
+        <v>46153</v>
       </c>
       <c r="F74" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G74" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H74" s="6" t="s">
         <v>23</v>
@@ -4738,22 +4759,22 @@
         <v>23</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K74" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="M74" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>23</v>
@@ -4782,13 +4803,13 @@
         <v>46167</v>
       </c>
       <c r="E75" s="7">
-        <v>46119</v>
+        <v>46127</v>
       </c>
       <c r="F75" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G75" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H75" s="6" t="s">
         <v>23</v>
@@ -4797,22 +4818,22 @@
         <v>23</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K75" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O75" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>23</v>
@@ -4824,7 +4845,7 @@
         <v>29</v>
       </c>
       <c r="S75" s="9">
-        <v>670</v>
+        <v>650</v>
       </c>
     </row>
     <row r="76" ht="23" customHeight="1">
@@ -4841,13 +4862,13 @@
         <v>46167</v>
       </c>
       <c r="E76" s="7">
-        <v>46113</v>
+        <v>46119</v>
       </c>
       <c r="F76" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G76" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H76" s="6" t="s">
         <v>23</v>
@@ -4856,22 +4877,22 @@
         <v>23</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K76" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="M76" s="6" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>23</v>
@@ -4883,7 +4904,7 @@
         <v>29</v>
       </c>
       <c r="S76" s="9">
-        <v>680</v>
+        <v>650</v>
       </c>
     </row>
     <row r="77" ht="23" customHeight="1">
@@ -4900,13 +4921,13 @@
         <v>46167</v>
       </c>
       <c r="E77" s="7">
-        <v>46119</v>
+        <v>46092</v>
       </c>
       <c r="F77" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G77" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H77" s="6" t="s">
         <v>23</v>
@@ -4915,22 +4936,22 @@
         <v>23</v>
       </c>
       <c r="J77" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K77" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="M77" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O77" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P77" s="6" t="s">
         <v>23</v>
@@ -4942,7 +4963,7 @@
         <v>29</v>
       </c>
       <c r="S77" s="9">
-        <v>680</v>
+        <v>650</v>
       </c>
     </row>
     <row r="78" ht="23" customHeight="1">
@@ -4962,10 +4983,10 @@
         <v>46119</v>
       </c>
       <c r="F78" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G78" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H78" s="6" t="s">
         <v>23</v>
@@ -4974,22 +4995,22 @@
         <v>23</v>
       </c>
       <c r="J78" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K78" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L78" s="6" t="s">
-        <v>32</v>
+        <v>132</v>
       </c>
       <c r="M78" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>23</v>
@@ -4998,10 +5019,10 @@
         <v>37</v>
       </c>
       <c r="R78" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S78" s="9">
-        <v>680</v>
+        <v>670</v>
       </c>
     </row>
     <row r="79" ht="23" customHeight="1">
@@ -5018,13 +5039,13 @@
         <v>46167</v>
       </c>
       <c r="E79" s="7">
-        <v>46141</v>
+        <v>46113</v>
       </c>
       <c r="F79" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G79" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H79" s="6" t="s">
         <v>23</v>
@@ -5033,22 +5054,22 @@
         <v>23</v>
       </c>
       <c r="J79" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="K79" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L79" s="6" t="s">
-        <v>98</v>
+        <v>44</v>
       </c>
       <c r="M79" s="6" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="N79" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O79" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P79" s="6" t="s">
         <v>23</v>
@@ -5057,7 +5078,7 @@
         <v>37</v>
       </c>
       <c r="R79" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S79" s="9">
         <v>680</v>
@@ -5077,13 +5098,13 @@
         <v>46167</v>
       </c>
       <c r="E80" s="7">
-        <v>46099</v>
+        <v>46119</v>
       </c>
       <c r="F80" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G80" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>23</v>
@@ -5092,22 +5113,22 @@
         <v>23</v>
       </c>
       <c r="J80" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K80" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L80" s="6" t="s">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="M80" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>23</v>
@@ -5116,10 +5137,10 @@
         <v>37</v>
       </c>
       <c r="R80" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="S80" s="9">
-        <v>700</v>
+        <v>680</v>
       </c>
     </row>
     <row r="81" ht="23" customHeight="1">
@@ -5136,13 +5157,13 @@
         <v>46167</v>
       </c>
       <c r="E81" s="7">
-        <v>46160</v>
+        <v>46119</v>
       </c>
       <c r="F81" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G81" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H81" s="6" t="s">
         <v>23</v>
@@ -5151,34 +5172,34 @@
         <v>23</v>
       </c>
       <c r="J81" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K81" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="M81" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N81" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O81" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P81" s="6" t="s">
-        <v>135</v>
+        <v>23</v>
       </c>
       <c r="Q81" s="6" t="s">
         <v>37</v>
       </c>
       <c r="R81" s="6" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="S81" s="9">
-        <v>1200</v>
+        <v>680</v>
       </c>
     </row>
     <row r="82" ht="23" customHeight="1">
@@ -5195,13 +5216,13 @@
         <v>46167</v>
       </c>
       <c r="E82" s="7">
-        <v>46160</v>
+        <v>46141</v>
       </c>
       <c r="F82" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G82" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H82" s="6" t="s">
         <v>23</v>
@@ -5216,28 +5237,28 @@
         <v>23</v>
       </c>
       <c r="L82" s="6" t="s">
-        <v>137</v>
+        <v>96</v>
       </c>
       <c r="M82" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>135</v>
+        <v>23</v>
       </c>
       <c r="Q82" s="6" t="s">
         <v>37</v>
       </c>
       <c r="R82" s="6" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="S82" s="9">
-        <v>1200</v>
+        <v>680</v>
       </c>
     </row>
     <row r="83" ht="23" customHeight="1">
@@ -5248,43 +5269,43 @@
         <v>46167</v>
       </c>
       <c r="C83" s="7">
-        <v>46113</v>
+        <v>46167</v>
       </c>
       <c r="D83" s="7">
-        <v>46150</v>
+        <v>46167</v>
       </c>
       <c r="E83" s="7">
-        <v>46149</v>
+        <v>46164</v>
       </c>
       <c r="F83" s="8">
-        <v>-13</v>
+        <v>3</v>
       </c>
       <c r="G83" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I83" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J83" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K83" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L83" s="6" t="s">
-        <v>139</v>
+        <v>98</v>
       </c>
       <c r="M83" s="6" t="s">
-        <v>140</v>
+        <v>23</v>
       </c>
       <c r="N83" s="6" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="O83" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P83" s="6" t="s">
         <v>23</v>
@@ -5293,69 +5314,305 @@
         <v>37</v>
       </c>
       <c r="R83" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="S83" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="84" ht="23" customHeight="1">
+      <c r="A84" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B84" s="7">
+        <v>46167</v>
+      </c>
+      <c r="C84" s="7">
+        <v>46167</v>
+      </c>
+      <c r="D84" s="7">
+        <v>46167</v>
+      </c>
+      <c r="E84" s="7">
+        <v>46099</v>
+      </c>
+      <c r="F84" s="8">
+        <v>3</v>
+      </c>
+      <c r="G84" s="8">
+        <v>3</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L84" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="M84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N84" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="O84" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="P84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q84" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R84" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="S84" s="9">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="85" ht="23" customHeight="1">
+      <c r="A85" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B85" s="7">
+        <v>46167</v>
+      </c>
+      <c r="C85" s="7">
+        <v>46167</v>
+      </c>
+      <c r="D85" s="7">
+        <v>46167</v>
+      </c>
+      <c r="E85" s="7">
+        <v>46160</v>
+      </c>
+      <c r="F85" s="8">
+        <v>3</v>
+      </c>
+      <c r="G85" s="8">
+        <v>3</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="K85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L85" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="M85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N85" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="O85" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="P85" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q85" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R85" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="S85" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="86" ht="23" customHeight="1">
+      <c r="A86" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B86" s="7">
+        <v>46167</v>
+      </c>
+      <c r="C86" s="7">
+        <v>46167</v>
+      </c>
+      <c r="D86" s="7">
+        <v>46167</v>
+      </c>
+      <c r="E86" s="7">
+        <v>46160</v>
+      </c>
+      <c r="F86" s="8">
+        <v>3</v>
+      </c>
+      <c r="G86" s="8">
+        <v>3</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="K86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L86" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="M86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N86" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="O86" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="P86" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q86" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R86" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="S86" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="87" ht="23" customHeight="1">
+      <c r="A87" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B87" s="7">
+        <v>46167</v>
+      </c>
+      <c r="C87" s="7">
+        <v>46113</v>
+      </c>
+      <c r="D87" s="7">
+        <v>46150</v>
+      </c>
+      <c r="E87" s="7">
+        <v>46149</v>
+      </c>
+      <c r="F87" s="8">
+        <v>-14</v>
+      </c>
+      <c r="G87" s="8">
+        <v>3</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L87" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="M87" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="N87" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O87" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="P87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q87" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R87" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="S83" s="9">
+      <c r="S87" s="9">
         <v>4400</v>
       </c>
     </row>
-    <row r="84" ht="23" customHeight="1">
-      <c r="A84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B84" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C84" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D84" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E84" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="F84" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G84" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="I84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="J84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="K84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="L84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="M84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="N84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="O84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="P84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="R84" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="S84" s="13">
-        <f>SUM(S6:S83)</f>
+    <row r="88" ht="23" customHeight="1">
+      <c r="A88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B88" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C88" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D88" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E88" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F88" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="G88" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="J88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="L88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="M88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="N88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="O88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="P88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="R88" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S88" s="13">
+        <f>SUM(S6:S87)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CONTAS-A-RECEBER spreadsheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/CONTAS-A-RECEBER.xlsx
+++ b/planilhas/CONTAS-A-RECEBER.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="159">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -40,7 +40,7 @@
     </r>
   </si>
   <si>
-    <t>Relatório exportado em segunda-feira, 25 de maio de 2026 por KAROL MEDEIROS</t>
+    <t>Relatório exportado em terça-feira, 26 de maio de 2026 por KAROL MEDEIROS</t>
   </si>
   <si>
     <t>Conta de Recebimento</t>
@@ -235,153 +235,153 @@
     <t>FA-11557</t>
   </si>
   <si>
-    <t>FA-11471</t>
+    <t>FA-11478</t>
+  </si>
+  <si>
+    <t>FA-11614</t>
+  </si>
+  <si>
+    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11453</t>
+  </si>
+  <si>
+    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
+  </si>
+  <si>
+    <t>FA-11390</t>
+  </si>
+  <si>
+    <t>FA-11458</t>
   </si>
   <si>
     <t>YAGO ELIAS COSTA BATISTA</t>
   </si>
   <si>
+    <t>FA-11615</t>
+  </si>
+  <si>
+    <t>FA-11396</t>
+  </si>
+  <si>
+    <t>FA-11525</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11559</t>
+  </si>
+  <si>
+    <t>FA-11497</t>
+  </si>
+  <si>
+    <t>ANDRE CAVALCANTI DA FE</t>
+  </si>
+  <si>
+    <t>FA-11466</t>
+  </si>
+  <si>
+    <t>FA-11474</t>
+  </si>
+  <si>
+    <t>FA-11481</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11560</t>
+  </si>
+  <si>
+    <t>DIEGO TAYAO DANTAS</t>
+  </si>
+  <si>
+    <t>FA-11402</t>
+  </si>
+  <si>
+    <t>FA-11616</t>
+  </si>
+  <si>
+    <t>FA-11620</t>
+  </si>
+  <si>
+    <t>FA-11675</t>
+  </si>
+  <si>
+    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
+  </si>
+  <si>
+    <t>FA-11483</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11561</t>
+  </si>
+  <si>
+    <t>ELSON VIEIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11484</t>
+  </si>
+  <si>
+    <t>FA-11479</t>
+  </si>
+  <si>
+    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11461</t>
+  </si>
+  <si>
+    <t>FA-11279</t>
+  </si>
+  <si>
+    <t>FELIPE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11476</t>
+  </si>
+  <si>
+    <t>FA-11674</t>
+  </si>
+  <si>
+    <t>FA-11611</t>
+  </si>
+  <si>
+    <t>M&amp;S DO TRABALHO</t>
+  </si>
+  <si>
+    <t>FA-11496</t>
+  </si>
+  <si>
+    <t>FA-11464</t>
+  </si>
+  <si>
+    <t>FA-11690</t>
+  </si>
+  <si>
+    <t>FA-11667</t>
+  </si>
+  <si>
+    <t>ND-11699</t>
+  </si>
+  <si>
+    <t>ROSSILY PEREIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>ND-11700</t>
+  </si>
+  <si>
+    <t>FA-11399</t>
+  </si>
+  <si>
     <t>FA-11473</t>
   </si>
   <si>
-    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
-  </si>
-  <si>
-    <t>FA-11478</t>
-  </si>
-  <si>
-    <t>FA-11614</t>
-  </si>
-  <si>
-    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11453</t>
-  </si>
-  <si>
-    <t>FA-11390</t>
-  </si>
-  <si>
-    <t>FA-11458</t>
-  </si>
-  <si>
-    <t>FA-11615</t>
-  </si>
-  <si>
-    <t>FA-11396</t>
-  </si>
-  <si>
-    <t>FA-11525</t>
-  </si>
-  <si>
-    <t>ROBERTO MURATORI</t>
-  </si>
-  <si>
-    <t>FA-11559</t>
-  </si>
-  <si>
-    <t>FA-11497</t>
-  </si>
-  <si>
-    <t>ANDRE CAVALCANTI DA FE</t>
-  </si>
-  <si>
-    <t>FA-11466</t>
-  </si>
-  <si>
-    <t>FA-11474</t>
-  </si>
-  <si>
-    <t>FA-11560</t>
-  </si>
-  <si>
-    <t>DIEGO TAYAO DANTAS</t>
-  </si>
-  <si>
-    <t>FA-11481</t>
-  </si>
-  <si>
-    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
-  </si>
-  <si>
-    <t>FA-11402</t>
-  </si>
-  <si>
-    <t>FA-11616</t>
-  </si>
-  <si>
-    <t>FA-11482</t>
-  </si>
-  <si>
-    <t>FA-11620</t>
-  </si>
-  <si>
-    <t>FA-11484</t>
-  </si>
-  <si>
-    <t>FA-11675</t>
-  </si>
-  <si>
-    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
-  </si>
-  <si>
-    <t>FA-11483</t>
-  </si>
-  <si>
-    <t>LUCAS NAJA MOURA RODRIGUES</t>
-  </si>
-  <si>
-    <t>FA-11561</t>
-  </si>
-  <si>
-    <t>ELSON VIEIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11479</t>
-  </si>
-  <si>
-    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11461</t>
-  </si>
-  <si>
-    <t>FA-11279</t>
-  </si>
-  <si>
-    <t>FELIPE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11476</t>
-  </si>
-  <si>
-    <t>FA-11674</t>
-  </si>
-  <si>
-    <t>FA-11611</t>
-  </si>
-  <si>
-    <t>M&amp;S DO TRABALHO</t>
-  </si>
-  <si>
-    <t>FA-11496</t>
-  </si>
-  <si>
-    <t>FA-11464</t>
-  </si>
-  <si>
-    <t>FA-11690</t>
-  </si>
-  <si>
-    <t>FA-11667</t>
-  </si>
-  <si>
-    <t>FA-11399</t>
-  </si>
-  <si>
-    <t>HOJE</t>
-  </si>
-  <si>
     <t>FA-11480</t>
   </si>
   <si>
@@ -397,15 +397,12 @@
     <t>FA-11668</t>
   </si>
   <si>
+    <t>FA-11617</t>
+  </si>
+  <si>
     <t>FA-11494</t>
   </si>
   <si>
-    <t>ROSSILY PEREIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11617</t>
-  </si>
-  <si>
     <t>FA-11683</t>
   </si>
   <si>
@@ -418,15 +415,15 @@
     <t>FA-11488</t>
   </si>
   <si>
+    <t>FA-11621</t>
+  </si>
+  <si>
     <t>FA-11504</t>
   </si>
   <si>
     <t>WESCLY JEAN DE MEDEIROS</t>
   </si>
   <si>
-    <t>FA-11621</t>
-  </si>
-  <si>
     <t>FA-11656</t>
   </si>
   <si>
@@ -439,24 +436,24 @@
     <t>RAYANE ROBERTA DA SILVA</t>
   </si>
   <si>
+    <t>FA-11564</t>
+  </si>
+  <si>
+    <t>FA-11489</t>
+  </si>
+  <si>
+    <t>FA-11691</t>
+  </si>
+  <si>
+    <t>FA-11676</t>
+  </si>
+  <si>
     <t>FA-11412</t>
   </si>
   <si>
     <t>FA-11491</t>
   </si>
   <si>
-    <t>FA-11691</t>
-  </si>
-  <si>
-    <t>FA-11564</t>
-  </si>
-  <si>
-    <t>FA-11489</t>
-  </si>
-  <si>
-    <t>FA-11676</t>
-  </si>
-  <si>
     <t>FA-11329</t>
   </si>
   <si>
@@ -478,6 +475,15 @@
     <t>ELIONILSON CORDEIRO BARBOSA</t>
   </si>
   <si>
+    <t>FA-11644</t>
+  </si>
+  <si>
+    <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
+  </si>
+  <si>
+    <t>PÚBLICO</t>
+  </si>
+  <si>
     <t>Z. FROTA INVESTIDORES - LUZ DIVINA</t>
   </si>
   <si>
@@ -494,15 +500,6 @@
   </si>
   <si>
     <t>TANIELLE GLAUCIANA SOUZA DA SILVA</t>
-  </si>
-  <si>
-    <t>PÚBLICO</t>
-  </si>
-  <si>
-    <t>FA-11644</t>
-  </si>
-  <si>
-    <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
   </si>
   <si>
     <t>FA-11613</t>
@@ -771,10 +768,10 @@
         <v>23</v>
       </c>
       <c r="F6" s="8">
-        <v>-49</v>
+        <v>-50</v>
       </c>
       <c r="G6" s="8">
-        <v>-35</v>
+        <v>-36</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>24</v>
@@ -830,10 +827,10 @@
         <v>23</v>
       </c>
       <c r="F7" s="8">
-        <v>-42</v>
+        <v>-43</v>
       </c>
       <c r="G7" s="8">
-        <v>-33</v>
+        <v>-34</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>24</v>
@@ -889,10 +886,10 @@
         <v>23</v>
       </c>
       <c r="F8" s="8">
-        <v>-42</v>
+        <v>-43</v>
       </c>
       <c r="G8" s="8">
-        <v>-31</v>
+        <v>-32</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>24</v>
@@ -948,10 +945,10 @@
         <v>46127</v>
       </c>
       <c r="F9" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G9" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>35</v>
@@ -1007,10 +1004,10 @@
         <v>46097</v>
       </c>
       <c r="F10" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G10" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>35</v>
@@ -1066,10 +1063,10 @@
         <v>23</v>
       </c>
       <c r="F11" s="8">
-        <v>-35</v>
+        <v>-36</v>
       </c>
       <c r="G11" s="8">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>24</v>
@@ -1125,10 +1122,10 @@
         <v>23</v>
       </c>
       <c r="F12" s="8">
-        <v>-56</v>
+        <v>-57</v>
       </c>
       <c r="G12" s="8">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>24</v>
@@ -1184,10 +1181,10 @@
         <v>23</v>
       </c>
       <c r="F13" s="8">
-        <v>-42</v>
+        <v>-43</v>
       </c>
       <c r="G13" s="8">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>24</v>
@@ -1243,10 +1240,10 @@
         <v>46141</v>
       </c>
       <c r="F14" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G14" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>35</v>
@@ -1302,10 +1299,10 @@
         <v>23</v>
       </c>
       <c r="F15" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G15" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>35</v>
@@ -1361,10 +1358,10 @@
         <v>23</v>
       </c>
       <c r="F16" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G16" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>35</v>
@@ -1420,10 +1417,10 @@
         <v>46097</v>
       </c>
       <c r="F17" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G17" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>35</v>
@@ -1479,10 +1476,10 @@
         <v>23</v>
       </c>
       <c r="F18" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G18" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>35</v>
@@ -1538,10 +1535,10 @@
         <v>46141</v>
       </c>
       <c r="F19" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G19" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>35</v>
@@ -1597,10 +1594,10 @@
         <v>23</v>
       </c>
       <c r="F20" s="8">
-        <v>-35</v>
+        <v>-36</v>
       </c>
       <c r="G20" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>24</v>
@@ -1656,10 +1653,10 @@
         <v>23</v>
       </c>
       <c r="F21" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G21" s="8">
-        <v>-20</v>
+        <v>-21</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>35</v>
@@ -1715,10 +1712,10 @@
         <v>46148</v>
       </c>
       <c r="F22" s="8">
-        <v>-25</v>
+        <v>-26</v>
       </c>
       <c r="G22" s="8">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>35</v>
@@ -1774,10 +1771,10 @@
         <v>23</v>
       </c>
       <c r="F23" s="8">
-        <v>-42</v>
+        <v>-43</v>
       </c>
       <c r="G23" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>24</v>
@@ -1833,10 +1830,10 @@
         <v>23</v>
       </c>
       <c r="F24" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G24" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>35</v>
@@ -1892,10 +1889,10 @@
         <v>46153</v>
       </c>
       <c r="F25" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G25" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>35</v>
@@ -1951,10 +1948,10 @@
         <v>23</v>
       </c>
       <c r="F26" s="8">
-        <v>-229</v>
+        <v>-230</v>
       </c>
       <c r="G26" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>64</v>
@@ -2010,10 +2007,10 @@
         <v>46097</v>
       </c>
       <c r="F27" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G27" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>35</v>
@@ -2069,10 +2066,10 @@
         <v>46141</v>
       </c>
       <c r="F28" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G28" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>35</v>
@@ -2128,10 +2125,10 @@
         <v>46119</v>
       </c>
       <c r="F29" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G29" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>35</v>
@@ -2146,10 +2143,10 @@
         <v>23</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="N29" s="6" t="s">
         <v>27</v>
@@ -2164,10 +2161,10 @@
         <v>37</v>
       </c>
       <c r="R29" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S29" s="9">
-        <v>600</v>
+        <v>680</v>
       </c>
     </row>
     <row r="30" ht="23" customHeight="1">
@@ -2175,19 +2172,19 @@
         <v>22</v>
       </c>
       <c r="B30" s="7">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="C30" s="7">
-        <v>46153</v>
+        <v>46146</v>
       </c>
       <c r="D30" s="7">
-        <v>46153</v>
-      </c>
-      <c r="E30" s="7">
-        <v>46119</v>
+        <v>46146</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F30" s="8">
-        <v>-14</v>
+        <v>-22</v>
       </c>
       <c r="G30" s="8">
         <v>-14</v>
@@ -2199,16 +2196,16 @@
         <v>35</v>
       </c>
       <c r="J30" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L30" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K30" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L30" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="M30" s="6" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="N30" s="6" t="s">
         <v>27</v>
@@ -2220,13 +2217,13 @@
         <v>23</v>
       </c>
       <c r="Q30" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R30" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S30" s="9">
-        <v>650</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" ht="23" customHeight="1">
@@ -2234,40 +2231,40 @@
         <v>22</v>
       </c>
       <c r="B31" s="7">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="C31" s="7">
-        <v>46153</v>
+        <v>46132</v>
       </c>
       <c r="D31" s="7">
-        <v>46153</v>
-      </c>
-      <c r="E31" s="7">
-        <v>46119</v>
+        <v>46132</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F31" s="8">
-        <v>-14</v>
+        <v>-36</v>
       </c>
       <c r="G31" s="8">
         <v>-14</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>35</v>
       </c>
       <c r="J31" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="K31" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L31" s="6" t="s">
-        <v>31</v>
-      </c>
       <c r="M31" s="6" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="N31" s="6" t="s">
         <v>27</v>
@@ -2279,13 +2276,13 @@
         <v>23</v>
       </c>
       <c r="Q31" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S31" s="9">
-        <v>680</v>
+        <v>317.54</v>
       </c>
     </row>
     <row r="32" ht="23" customHeight="1">
@@ -2293,25 +2290,25 @@
         <v>22</v>
       </c>
       <c r="B32" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="C32" s="7">
-        <v>46146</v>
+        <v>46132</v>
       </c>
       <c r="D32" s="7">
-        <v>46146</v>
+        <v>46132</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F32" s="8">
-        <v>-21</v>
+        <v>-36</v>
       </c>
       <c r="G32" s="8">
         <v>-13</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>35</v>
@@ -2323,7 +2320,7 @@
         <v>23</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>23</v>
@@ -2344,7 +2341,7 @@
         <v>29</v>
       </c>
       <c r="S32" s="9">
-        <v>280</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" ht="23" customHeight="1">
@@ -2352,40 +2349,40 @@
         <v>22</v>
       </c>
       <c r="B33" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="C33" s="7">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="D33" s="7">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F33" s="8">
-        <v>-35</v>
+        <v>-29</v>
       </c>
       <c r="G33" s="8">
         <v>-13</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="I33" s="6" t="s">
         <v>35</v>
       </c>
       <c r="J33" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="K33" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="M33" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N33" s="6" t="s">
         <v>27</v>
@@ -2403,7 +2400,7 @@
         <v>29</v>
       </c>
       <c r="S33" s="9">
-        <v>317.54</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" ht="23" customHeight="1">
@@ -2414,22 +2411,22 @@
         <v>46155</v>
       </c>
       <c r="C34" s="7">
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="D34" s="7">
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F34" s="8">
-        <v>-35</v>
+        <v>-15</v>
       </c>
       <c r="G34" s="8">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>35</v>
@@ -2441,7 +2438,7 @@
         <v>23</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="M34" s="6" t="s">
         <v>23</v>
@@ -2462,7 +2459,7 @@
         <v>29</v>
       </c>
       <c r="S34" s="9">
-        <v>140</v>
+        <v>530</v>
       </c>
     </row>
     <row r="35" ht="23" customHeight="1">
@@ -2470,19 +2467,19 @@
         <v>22</v>
       </c>
       <c r="B35" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="C35" s="7">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="D35" s="7">
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F35" s="8">
-        <v>-28</v>
+        <v>-22</v>
       </c>
       <c r="G35" s="8">
         <v>-12</v>
@@ -2500,10 +2497,10 @@
         <v>23</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="N35" s="6" t="s">
         <v>27</v>
@@ -2521,7 +2518,7 @@
         <v>29</v>
       </c>
       <c r="S35" s="9">
-        <v>250</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1">
@@ -2529,22 +2526,22 @@
         <v>22</v>
       </c>
       <c r="B36" s="7">
-        <v>46155</v>
+        <v>46160</v>
       </c>
       <c r="C36" s="7">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="D36" s="7">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F36" s="8">
-        <v>-14</v>
+        <v>-8</v>
       </c>
       <c r="G36" s="8">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>35</v>
@@ -2553,13 +2550,13 @@
         <v>35</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>73</v>
+        <v>23</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>23</v>
@@ -2580,7 +2577,7 @@
         <v>29</v>
       </c>
       <c r="S36" s="9">
-        <v>530</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="37" ht="23" customHeight="1">
@@ -2588,22 +2585,22 @@
         <v>22</v>
       </c>
       <c r="B37" s="7">
-        <v>46156</v>
+        <v>46160</v>
       </c>
       <c r="C37" s="7">
-        <v>46146</v>
+        <v>46082</v>
       </c>
       <c r="D37" s="7">
-        <v>46146</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>23</v>
+        <v>46160</v>
+      </c>
+      <c r="E37" s="7">
+        <v>46097</v>
       </c>
       <c r="F37" s="8">
-        <v>-21</v>
+        <v>-8</v>
       </c>
       <c r="G37" s="8">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>35</v>
@@ -2612,13 +2609,13 @@
         <v>35</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>23</v>
@@ -2633,13 +2630,13 @@
         <v>23</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="R37" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S37" s="9">
-        <v>130</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="38" ht="23" customHeight="1">
@@ -2655,14 +2652,14 @@
       <c r="D38" s="7">
         <v>46160</v>
       </c>
-      <c r="E38" s="7" t="s">
-        <v>23</v>
+      <c r="E38" s="7">
+        <v>46127</v>
       </c>
       <c r="F38" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G38" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>35</v>
@@ -2671,16 +2668,16 @@
         <v>35</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="N38" s="6" t="s">
         <v>27</v>
@@ -2692,13 +2689,13 @@
         <v>23</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R38" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S38" s="9">
-        <v>97.5</v>
+        <v>172</v>
       </c>
     </row>
     <row r="39" ht="23" customHeight="1">
@@ -2709,19 +2706,19 @@
         <v>46160</v>
       </c>
       <c r="C39" s="7">
-        <v>46082</v>
+        <v>46160</v>
       </c>
       <c r="D39" s="7">
         <v>46160</v>
       </c>
       <c r="E39" s="7">
-        <v>46097</v>
+        <v>46141</v>
       </c>
       <c r="F39" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G39" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>35</v>
@@ -2730,13 +2727,13 @@
         <v>35</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="K39" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>23</v>
@@ -2751,13 +2748,13 @@
         <v>23</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R39" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S39" s="9">
-        <v>146.55</v>
+        <v>310</v>
       </c>
     </row>
     <row r="40" ht="23" customHeight="1">
@@ -2768,37 +2765,37 @@
         <v>46160</v>
       </c>
       <c r="C40" s="7">
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="D40" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E40" s="7">
-        <v>46127</v>
+        <v>46132</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F40" s="8">
-        <v>-7</v>
+        <v>-36</v>
       </c>
       <c r="G40" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I40" s="6" t="s">
         <v>35</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>80</v>
+        <v>23</v>
       </c>
       <c r="N40" s="6" t="s">
         <v>27</v>
@@ -2810,13 +2807,13 @@
         <v>23</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R40" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S40" s="9">
-        <v>172</v>
+        <v>350</v>
       </c>
     </row>
     <row r="41" ht="23" customHeight="1">
@@ -2827,19 +2824,19 @@
         <v>46160</v>
       </c>
       <c r="C41" s="7">
-        <v>46160</v>
+        <v>46146</v>
       </c>
       <c r="D41" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E41" s="7">
-        <v>46141</v>
+        <v>46146</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F41" s="8">
-        <v>-7</v>
+        <v>-22</v>
       </c>
       <c r="G41" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>35</v>
@@ -2848,16 +2845,16 @@
         <v>35</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K41" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="N41" s="6" t="s">
         <v>27</v>
@@ -2869,13 +2866,13 @@
         <v>23</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R41" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S41" s="9">
-        <v>310</v>
+        <v>450</v>
       </c>
     </row>
     <row r="42" ht="23" customHeight="1">
@@ -2886,37 +2883,37 @@
         <v>46160</v>
       </c>
       <c r="C42" s="7">
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="D42" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>23</v>
+        <v>46160</v>
+      </c>
+      <c r="E42" s="7">
+        <v>46119</v>
       </c>
       <c r="F42" s="8">
-        <v>-35</v>
+        <v>-8</v>
       </c>
       <c r="G42" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="I42" s="6" t="s">
         <v>35</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K42" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="N42" s="6" t="s">
         <v>27</v>
@@ -2928,13 +2925,13 @@
         <v>23</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R42" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S42" s="9">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="43" ht="23" customHeight="1">
@@ -2945,19 +2942,19 @@
         <v>46160</v>
       </c>
       <c r="C43" s="7">
-        <v>46146</v>
+        <v>46160</v>
       </c>
       <c r="D43" s="7">
-        <v>46146</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>23</v>
+        <v>46160</v>
+      </c>
+      <c r="E43" s="7">
+        <v>46119</v>
       </c>
       <c r="F43" s="8">
-        <v>-21</v>
+        <v>-8</v>
       </c>
       <c r="G43" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>35</v>
@@ -2972,10 +2969,10 @@
         <v>23</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="N43" s="6" t="s">
         <v>27</v>
@@ -2987,13 +2984,13 @@
         <v>23</v>
       </c>
       <c r="Q43" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R43" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S43" s="9">
-        <v>450</v>
+        <v>620</v>
       </c>
     </row>
     <row r="44" ht="23" customHeight="1">
@@ -3010,13 +3007,13 @@
         <v>46160</v>
       </c>
       <c r="E44" s="7">
-        <v>46119</v>
+        <v>46141</v>
       </c>
       <c r="F44" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G44" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>35</v>
@@ -3025,16 +3022,16 @@
         <v>35</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K44" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="N44" s="6" t="s">
         <v>27</v>
@@ -3052,7 +3049,7 @@
         <v>29</v>
       </c>
       <c r="S44" s="9">
-        <v>600</v>
+        <v>620</v>
       </c>
     </row>
     <row r="45" ht="23" customHeight="1">
@@ -3069,13 +3066,13 @@
         <v>46160</v>
       </c>
       <c r="E45" s="7">
-        <v>46141</v>
+        <v>46112</v>
       </c>
       <c r="F45" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G45" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>35</v>
@@ -3084,16 +3081,16 @@
         <v>35</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="N45" s="6" t="s">
         <v>27</v>
@@ -3111,7 +3108,7 @@
         <v>29</v>
       </c>
       <c r="S45" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="46" ht="23" customHeight="1">
@@ -3128,13 +3125,13 @@
         <v>46160</v>
       </c>
       <c r="E46" s="7">
-        <v>46119</v>
+        <v>46150</v>
       </c>
       <c r="F46" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G46" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>35</v>
@@ -3143,16 +3140,16 @@
         <v>35</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="N46" s="6" t="s">
         <v>27</v>
@@ -3167,10 +3164,10 @@
         <v>37</v>
       </c>
       <c r="R46" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S46" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="47" ht="23" customHeight="1">
@@ -3187,13 +3184,13 @@
         <v>46160</v>
       </c>
       <c r="E47" s="7">
-        <v>46112</v>
+        <v>46153</v>
       </c>
       <c r="F47" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G47" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>35</v>
@@ -3208,7 +3205,7 @@
         <v>23</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="M47" s="6" t="s">
         <v>23</v>
@@ -3229,7 +3226,7 @@
         <v>29</v>
       </c>
       <c r="S47" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="48" ht="23" customHeight="1">
@@ -3246,13 +3243,13 @@
         <v>46160</v>
       </c>
       <c r="E48" s="7">
-        <v>46150</v>
+        <v>46164</v>
       </c>
       <c r="F48" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G48" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>35</v>
@@ -3267,7 +3264,7 @@
         <v>23</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="M48" s="6" t="s">
         <v>23</v>
@@ -3285,10 +3282,10 @@
         <v>37</v>
       </c>
       <c r="R48" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S48" s="9">
-        <v>630</v>
+        <v>680</v>
       </c>
     </row>
     <row r="49" ht="23" customHeight="1">
@@ -3308,10 +3305,10 @@
         <v>46119</v>
       </c>
       <c r="F49" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G49" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>35</v>
@@ -3320,16 +3317,16 @@
         <v>35</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K49" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="N49" s="6" t="s">
         <v>27</v>
@@ -3347,7 +3344,7 @@
         <v>29</v>
       </c>
       <c r="S49" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="50" ht="23" customHeight="1">
@@ -3364,13 +3361,13 @@
         <v>46160</v>
       </c>
       <c r="E50" s="7">
-        <v>46153</v>
+        <v>46141</v>
       </c>
       <c r="F50" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G50" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H50" s="6" t="s">
         <v>35</v>
@@ -3379,13 +3376,13 @@
         <v>35</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K50" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>23</v>
@@ -3403,10 +3400,10 @@
         <v>37</v>
       </c>
       <c r="R50" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S50" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="51" ht="23" customHeight="1">
@@ -3426,10 +3423,10 @@
         <v>46119</v>
       </c>
       <c r="F51" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G51" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>35</v>
@@ -3438,7 +3435,7 @@
         <v>35</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="K51" s="6" t="s">
         <v>23</v>
@@ -3482,13 +3479,13 @@
         <v>46160</v>
       </c>
       <c r="E52" s="7">
-        <v>46164</v>
+        <v>46119</v>
       </c>
       <c r="F52" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G52" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>35</v>
@@ -3497,13 +3494,13 @@
         <v>35</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="K52" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="M52" s="6" t="s">
         <v>23</v>
@@ -3515,16 +3512,16 @@
         <v>27</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>37</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S52" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="53" ht="23" customHeight="1">
@@ -3532,19 +3529,19 @@
         <v>22</v>
       </c>
       <c r="B53" s="7">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="C53" s="7">
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="D53" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E53" s="7">
-        <v>46119</v>
+        <v>46139</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F53" s="8">
-        <v>-7</v>
+        <v>-29</v>
       </c>
       <c r="G53" s="8">
         <v>-7</v>
@@ -3556,13 +3553,13 @@
         <v>35</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="K53" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M53" s="6" t="s">
         <v>23</v>
@@ -3574,16 +3571,16 @@
         <v>27</v>
       </c>
       <c r="P53" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="Q53" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R53" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S53" s="9">
-        <v>680</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" ht="23" customHeight="1">
@@ -3591,7 +3588,7 @@
         <v>22</v>
       </c>
       <c r="B54" s="7">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="C54" s="7">
         <v>46160</v>
@@ -3599,11 +3596,11 @@
       <c r="D54" s="7">
         <v>46160</v>
       </c>
-      <c r="E54" s="7">
-        <v>46141</v>
+      <c r="E54" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F54" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G54" s="8">
         <v>-7</v>
@@ -3615,13 +3612,13 @@
         <v>35</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>23</v>
@@ -3636,13 +3633,13 @@
         <v>23</v>
       </c>
       <c r="Q54" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R54" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S54" s="9">
-        <v>680</v>
+        <v>130</v>
       </c>
     </row>
     <row r="55" ht="23" customHeight="1">
@@ -3650,19 +3647,19 @@
         <v>22</v>
       </c>
       <c r="B55" s="7">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="C55" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="D55" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E55" s="7">
-        <v>46119</v>
+        <v>46153</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F55" s="8">
-        <v>-7</v>
+        <v>-15</v>
       </c>
       <c r="G55" s="8">
         <v>-7</v>
@@ -3674,16 +3671,16 @@
         <v>35</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K55" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="N55" s="6" t="s">
         <v>27</v>
@@ -3692,16 +3689,16 @@
         <v>27</v>
       </c>
       <c r="P55" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="Q55" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R55" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S55" s="9">
-        <v>700</v>
+        <v>277.36</v>
       </c>
     </row>
     <row r="56" ht="23" customHeight="1">
@@ -3712,19 +3709,19 @@
         <v>46161</v>
       </c>
       <c r="C56" s="7">
-        <v>46139</v>
+        <v>46153</v>
       </c>
       <c r="D56" s="7">
-        <v>46139</v>
+        <v>46153</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F56" s="8">
-        <v>-28</v>
+        <v>-15</v>
       </c>
       <c r="G56" s="8">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>35</v>
@@ -3733,13 +3730,13 @@
         <v>35</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>23</v>
@@ -3751,16 +3748,16 @@
         <v>27</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="Q56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="R56" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S56" s="9">
-        <v>50</v>
+        <v>280</v>
       </c>
     </row>
     <row r="57" ht="23" customHeight="1">
@@ -3771,20 +3768,20 @@
         <v>46161</v>
       </c>
       <c r="C57" s="7">
-        <v>46160</v>
+        <v>46113</v>
       </c>
       <c r="D57" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E57" s="7" t="s">
-        <v>23</v>
+        <v>46150</v>
+      </c>
+      <c r="E57" s="7">
+        <v>46149</v>
       </c>
       <c r="F57" s="8">
+        <v>-18</v>
+      </c>
+      <c r="G57" s="8">
         <v>-7</v>
       </c>
-      <c r="G57" s="8">
-        <v>-6</v>
-      </c>
       <c r="H57" s="6" t="s">
         <v>35</v>
       </c>
@@ -3792,16 +3789,16 @@
         <v>35</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="N57" s="6" t="s">
         <v>27</v>
@@ -3813,13 +3810,13 @@
         <v>23</v>
       </c>
       <c r="Q57" s="6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="R57" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S57" s="9">
-        <v>130</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="58" ht="23" customHeight="1">
@@ -3827,40 +3824,40 @@
         <v>22</v>
       </c>
       <c r="B58" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="C58" s="7">
-        <v>46153</v>
+        <v>46125</v>
       </c>
       <c r="D58" s="7">
-        <v>46153</v>
+        <v>46125</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F58" s="8">
-        <v>-14</v>
+        <v>-43</v>
       </c>
       <c r="G58" s="8">
         <v>-6</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I58" s="6" t="s">
         <v>35</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K58" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="N58" s="6" t="s">
         <v>27</v>
@@ -3878,7 +3875,7 @@
         <v>32</v>
       </c>
       <c r="S58" s="9">
-        <v>277.36</v>
+        <v>50</v>
       </c>
     </row>
     <row r="59" ht="23" customHeight="1">
@@ -3886,19 +3883,19 @@
         <v>22</v>
       </c>
       <c r="B59" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="C59" s="7">
-        <v>46153</v>
+        <v>46146</v>
       </c>
       <c r="D59" s="7">
-        <v>46153</v>
+        <v>46146</v>
       </c>
       <c r="E59" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F59" s="8">
-        <v>-14</v>
+        <v>-22</v>
       </c>
       <c r="G59" s="8">
         <v>-6</v>
@@ -3910,16 +3907,16 @@
         <v>35</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K59" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="M59" s="6" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="N59" s="6" t="s">
         <v>27</v>
@@ -3934,10 +3931,10 @@
         <v>23</v>
       </c>
       <c r="R59" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S59" s="9">
-        <v>280</v>
+        <v>200</v>
       </c>
     </row>
     <row r="60" ht="23" customHeight="1">
@@ -3945,19 +3942,19 @@
         <v>22</v>
       </c>
       <c r="B60" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="C60" s="7">
-        <v>46113</v>
+        <v>46160</v>
       </c>
       <c r="D60" s="7">
-        <v>46150</v>
-      </c>
-      <c r="E60" s="7">
-        <v>46149</v>
+        <v>46160</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F60" s="8">
-        <v>-17</v>
+        <v>-8</v>
       </c>
       <c r="G60" s="8">
         <v>-6</v>
@@ -3969,16 +3966,16 @@
         <v>35</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K60" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>109</v>
+        <v>59</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="N60" s="6" t="s">
         <v>27</v>
@@ -3990,13 +3987,13 @@
         <v>23</v>
       </c>
       <c r="Q60" s="6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R60" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S60" s="9">
-        <v>2100</v>
+        <v>380</v>
       </c>
     </row>
     <row r="61" ht="23" customHeight="1">
@@ -4004,25 +4001,25 @@
         <v>22</v>
       </c>
       <c r="B61" s="7">
-        <v>46162</v>
+        <v>46164</v>
       </c>
       <c r="C61" s="7">
-        <v>46125</v>
+        <v>46160</v>
       </c>
       <c r="D61" s="7">
-        <v>46125</v>
+        <v>46160</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F61" s="8">
-        <v>-42</v>
+        <v>-8</v>
       </c>
       <c r="G61" s="8">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="I61" s="6" t="s">
         <v>35</v>
@@ -4034,7 +4031,7 @@
         <v>23</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="M61" s="6" t="s">
         <v>23</v>
@@ -4052,10 +4049,10 @@
         <v>23</v>
       </c>
       <c r="R61" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S61" s="9">
-        <v>50</v>
+        <v>290</v>
       </c>
     </row>
     <row r="62" ht="23" customHeight="1">
@@ -4063,22 +4060,22 @@
         <v>22</v>
       </c>
       <c r="B62" s="7">
-        <v>46162</v>
+        <v>46167</v>
       </c>
       <c r="C62" s="7">
-        <v>46146</v>
+        <v>46143</v>
       </c>
       <c r="D62" s="7">
-        <v>46146</v>
-      </c>
-      <c r="E62" s="7" t="s">
-        <v>23</v>
+        <v>46167</v>
+      </c>
+      <c r="E62" s="7">
+        <v>46153</v>
       </c>
       <c r="F62" s="8">
-        <v>-21</v>
+        <v>-1</v>
       </c>
       <c r="G62" s="8">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>35</v>
@@ -4093,10 +4090,10 @@
         <v>23</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="N62" s="6" t="s">
         <v>27</v>
@@ -4105,16 +4102,16 @@
         <v>27</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="Q62" s="6" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="R62" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S62" s="9">
-        <v>200</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" ht="23" customHeight="1">
@@ -4122,22 +4119,22 @@
         <v>22</v>
       </c>
       <c r="B63" s="7">
-        <v>46162</v>
+        <v>46167</v>
       </c>
       <c r="C63" s="7">
-        <v>46160</v>
+        <v>46143</v>
       </c>
       <c r="D63" s="7">
-        <v>46160</v>
-      </c>
-      <c r="E63" s="7" t="s">
-        <v>23</v>
+        <v>46167</v>
+      </c>
+      <c r="E63" s="7">
+        <v>46167</v>
       </c>
       <c r="F63" s="8">
-        <v>-7</v>
+        <v>-1</v>
       </c>
       <c r="G63" s="8">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>35</v>
@@ -4146,13 +4143,13 @@
         <v>35</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="M63" s="6" t="s">
         <v>23</v>
@@ -4167,13 +4164,13 @@
         <v>23</v>
       </c>
       <c r="Q63" s="6" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="R63" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S63" s="9">
-        <v>380</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64" ht="23" customHeight="1">
@@ -4181,22 +4178,22 @@
         <v>22</v>
       </c>
       <c r="B64" s="7">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="C64" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="D64" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F64" s="8">
-        <v>-7</v>
+        <v>-15</v>
       </c>
       <c r="G64" s="8">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>35</v>
@@ -4205,13 +4202,13 @@
         <v>35</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="M64" s="6" t="s">
         <v>23</v>
@@ -4232,7 +4229,7 @@
         <v>29</v>
       </c>
       <c r="S64" s="9">
-        <v>290</v>
+        <v>130</v>
       </c>
     </row>
     <row r="65" ht="23" customHeight="1">
@@ -4243,34 +4240,34 @@
         <v>46167</v>
       </c>
       <c r="C65" s="7">
-        <v>46153</v>
+        <v>46082</v>
       </c>
       <c r="D65" s="7">
-        <v>46153</v>
-      </c>
-      <c r="E65" s="7" t="s">
-        <v>23</v>
+        <v>46167</v>
+      </c>
+      <c r="E65" s="7">
+        <v>46097</v>
       </c>
       <c r="F65" s="8">
-        <v>-14</v>
+        <v>-1</v>
       </c>
       <c r="G65" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H65" s="6" t="s">
         <v>35</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="K65" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="M65" s="6" t="s">
         <v>23</v>
@@ -4279,19 +4276,19 @@
         <v>27</v>
       </c>
       <c r="O65" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P65" s="6" t="s">
         <v>23</v>
       </c>
       <c r="Q65" s="6" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="R65" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S65" s="9">
-        <v>130</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="66" ht="23" customHeight="1">
@@ -4302,55 +4299,55 @@
         <v>46167</v>
       </c>
       <c r="C66" s="7">
-        <v>46082</v>
+        <v>46153</v>
       </c>
       <c r="D66" s="7">
-        <v>46167</v>
-      </c>
-      <c r="E66" s="7">
-        <v>46097</v>
+        <v>46153</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F66" s="8">
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="G66" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="K66" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="M66" s="6" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>23</v>
       </c>
       <c r="Q66" s="6" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="R66" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S66" s="9">
-        <v>146.55</v>
+        <v>400</v>
       </c>
     </row>
     <row r="67" ht="23" customHeight="1">
@@ -4370,16 +4367,16 @@
         <v>46119</v>
       </c>
       <c r="F67" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G67" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J67" s="6" t="s">
         <v>116</v>
@@ -4388,16 +4385,16 @@
         <v>23</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="M67" s="6" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P67" s="6" t="s">
         <v>23</v>
@@ -4429,16 +4426,16 @@
         <v>46141</v>
       </c>
       <c r="F68" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G68" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J68" s="6" t="s">
         <v>117</v>
@@ -4453,10 +4450,10 @@
         <v>23</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>23</v>
@@ -4488,16 +4485,16 @@
         <v>46119</v>
       </c>
       <c r="F69" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G69" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J69" s="6" t="s">
         <v>118</v>
@@ -4506,16 +4503,16 @@
         <v>23</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O69" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P69" s="6" t="s">
         <v>23</v>
@@ -4547,16 +4544,16 @@
         <v>46141</v>
       </c>
       <c r="F70" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G70" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J70" s="6" t="s">
         <v>119</v>
@@ -4571,10 +4568,10 @@
         <v>87</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>23</v>
@@ -4606,16 +4603,16 @@
         <v>46163</v>
       </c>
       <c r="F71" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G71" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J71" s="6" t="s">
         <v>120</v>
@@ -4630,10 +4627,10 @@
         <v>23</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O71" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P71" s="6" t="s">
         <v>23</v>
@@ -4662,19 +4659,19 @@
         <v>46167</v>
       </c>
       <c r="E72" s="7">
-        <v>46119</v>
+        <v>46150</v>
       </c>
       <c r="F72" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G72" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J72" s="6" t="s">
         <v>121</v>
@@ -4683,19 +4680,19 @@
         <v>23</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>122</v>
+        <v>69</v>
       </c>
       <c r="M72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="Q72" s="6" t="s">
         <v>37</v>
@@ -4721,40 +4718,40 @@
         <v>46167</v>
       </c>
       <c r="E73" s="7">
-        <v>46150</v>
+        <v>46119</v>
       </c>
       <c r="F73" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G73" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>73</v>
+        <v>112</v>
       </c>
       <c r="M73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O73" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P73" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="Q73" s="6" t="s">
         <v>37</v>
@@ -4783,34 +4780,34 @@
         <v>46164</v>
       </c>
       <c r="F74" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G74" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J74" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L74" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="K74" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L74" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="M74" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>23</v>
@@ -4842,34 +4839,34 @@
         <v>46092</v>
       </c>
       <c r="F75" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G75" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K75" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O75" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>23</v>
@@ -4901,34 +4898,34 @@
         <v>46119</v>
       </c>
       <c r="F76" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G76" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K76" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M76" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>23</v>
@@ -4957,37 +4954,37 @@
         <v>46167</v>
       </c>
       <c r="E77" s="7">
-        <v>46127</v>
+        <v>46153</v>
       </c>
       <c r="F77" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G77" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J77" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K77" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>129</v>
+        <v>63</v>
       </c>
       <c r="M77" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O77" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P77" s="6" t="s">
         <v>23</v>
@@ -5016,37 +5013,37 @@
         <v>46167</v>
       </c>
       <c r="E78" s="7">
-        <v>46153</v>
+        <v>46127</v>
       </c>
       <c r="F78" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G78" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I78" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J78" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K78" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L78" s="6" t="s">
-        <v>63</v>
+        <v>129</v>
       </c>
       <c r="M78" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>23</v>
@@ -5078,34 +5075,34 @@
         <v>46160</v>
       </c>
       <c r="F79" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G79" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J79" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L79" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="K79" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L79" s="6" t="s">
-        <v>132</v>
-      </c>
       <c r="M79" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N79" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O79" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P79" s="6" t="s">
         <v>23</v>
@@ -5137,34 +5134,34 @@
         <v>46119</v>
       </c>
       <c r="F80" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G80" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J80" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L80" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="K80" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L80" s="6" t="s">
-        <v>134</v>
-      </c>
       <c r="M80" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>23</v>
@@ -5193,37 +5190,37 @@
         <v>46167</v>
       </c>
       <c r="E81" s="7">
-        <v>46113</v>
+        <v>46141</v>
       </c>
       <c r="F81" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G81" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J81" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K81" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="M81" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="N81" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O81" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P81" s="6" t="s">
         <v>23</v>
@@ -5232,7 +5229,7 @@
         <v>37</v>
       </c>
       <c r="R81" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="S81" s="9">
         <v>680</v>
@@ -5255,34 +5252,34 @@
         <v>46119</v>
       </c>
       <c r="F82" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G82" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I82" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J82" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K82" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L82" s="6" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="M82" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>23</v>
@@ -5291,7 +5288,7 @@
         <v>37</v>
       </c>
       <c r="R82" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="S82" s="9">
         <v>680</v>
@@ -5314,19 +5311,19 @@
         <v>46167</v>
       </c>
       <c r="F83" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G83" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I83" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J83" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K83" s="6" t="s">
         <v>23</v>
@@ -5338,10 +5335,10 @@
         <v>23</v>
       </c>
       <c r="N83" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O83" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P83" s="6" t="s">
         <v>23</v>
@@ -5370,37 +5367,37 @@
         <v>46167</v>
       </c>
       <c r="E84" s="7">
-        <v>46141</v>
+        <v>46164</v>
       </c>
       <c r="F84" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G84" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I84" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J84" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K84" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L84" s="6" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="M84" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>23</v>
@@ -5429,37 +5426,37 @@
         <v>46167</v>
       </c>
       <c r="E85" s="7">
-        <v>46119</v>
+        <v>46113</v>
       </c>
       <c r="F85" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G85" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I85" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J85" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K85" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L85" s="6" t="s">
-        <v>98</v>
+        <v>46</v>
       </c>
       <c r="M85" s="6" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="N85" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O85" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P85" s="6" t="s">
         <v>23</v>
@@ -5488,37 +5485,37 @@
         <v>46167</v>
       </c>
       <c r="E86" s="7">
-        <v>46164</v>
+        <v>46119</v>
       </c>
       <c r="F86" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G86" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I86" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J86" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K86" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L86" s="6" t="s">
-        <v>96</v>
+        <v>31</v>
       </c>
       <c r="M86" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P86" s="6" t="s">
         <v>23</v>
@@ -5550,34 +5547,34 @@
         <v>46099</v>
       </c>
       <c r="F87" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G87" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I87" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J87" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L87" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="K87" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L87" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="M87" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N87" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O87" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P87" s="6" t="s">
         <v>23</v>
@@ -5594,7 +5591,7 @@
     </row>
     <row r="88" ht="23" customHeight="1">
       <c r="A88" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B88" s="7">
         <v>46167</v>
@@ -5609,34 +5606,34 @@
         <v>46148</v>
       </c>
       <c r="F88" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G88" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I88" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J88" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L88" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="K88" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L88" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="M88" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P88" s="6" t="s">
         <v>23</v>
@@ -5653,7 +5650,7 @@
     </row>
     <row r="89" ht="23" customHeight="1">
       <c r="A89" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B89" s="7">
         <v>46167</v>
@@ -5668,34 +5665,34 @@
         <v>46129</v>
       </c>
       <c r="F89" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G89" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I89" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J89" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="K89" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L89" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="K89" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L89" s="6" t="s">
-        <v>147</v>
-      </c>
       <c r="M89" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N89" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O89" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>23</v>
@@ -5712,52 +5709,52 @@
     </row>
     <row r="90" ht="23" customHeight="1">
       <c r="A90" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B90" s="7">
+        <v>46167</v>
+      </c>
+      <c r="C90" s="7">
+        <v>46167</v>
+      </c>
+      <c r="D90" s="7">
+        <v>46167</v>
+      </c>
+      <c r="E90" s="7">
+        <v>46160</v>
+      </c>
+      <c r="F90" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G90" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L90" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="B90" s="7">
-        <v>46167</v>
-      </c>
-      <c r="C90" s="7">
-        <v>46167</v>
-      </c>
-      <c r="D90" s="7">
-        <v>46167</v>
-      </c>
-      <c r="E90" s="7">
-        <v>46148</v>
-      </c>
-      <c r="F90" s="8">
-        <v>0</v>
-      </c>
-      <c r="G90" s="8">
-        <v>0</v>
-      </c>
-      <c r="H90" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I90" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J90" s="6" t="s">
+      <c r="M90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N90" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O90" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P90" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="K90" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L90" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="M90" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N90" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="O90" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="P90" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="Q90" s="6" t="s">
         <v>37</v>
@@ -5771,7 +5768,7 @@
     </row>
     <row r="91" ht="23" customHeight="1">
       <c r="A91" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B91" s="7">
         <v>46167</v>
@@ -5786,16 +5783,16 @@
         <v>46148</v>
       </c>
       <c r="F91" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G91" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I91" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J91" s="6" t="s">
         <v>151</v>
@@ -5804,16 +5801,16 @@
         <v>23</v>
       </c>
       <c r="L91" s="6" t="s">
-        <v>56</v>
+        <v>152</v>
       </c>
       <c r="M91" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N91" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O91" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P91" s="6" t="s">
         <v>23</v>
@@ -5830,7 +5827,7 @@
     </row>
     <row r="92" ht="23" customHeight="1">
       <c r="A92" s="6" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="B92" s="7">
         <v>46167</v>
@@ -5842,40 +5839,40 @@
         <v>46167</v>
       </c>
       <c r="E92" s="7">
-        <v>46160</v>
+        <v>46148</v>
       </c>
       <c r="F92" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G92" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I92" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J92" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K92" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L92" s="6" t="s">
-        <v>153</v>
+        <v>56</v>
       </c>
       <c r="M92" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>154</v>
+        <v>23</v>
       </c>
       <c r="Q92" s="6" t="s">
         <v>37</v>
@@ -5904,37 +5901,37 @@
         <v>46160</v>
       </c>
       <c r="F93" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G93" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I93" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J93" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="K93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L93" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="K93" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L93" s="6" t="s">
-        <v>156</v>
-      </c>
       <c r="M93" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N93" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="O93" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P93" s="6" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="Q93" s="6" t="s">
         <v>37</v>
@@ -5963,34 +5960,34 @@
         <v>46149</v>
       </c>
       <c r="F94" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="G94" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H94" s="6" t="s">
         <v>35</v>
       </c>
       <c r="I94" s="6" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="J94" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="K94" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L94" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="K94" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L94" s="6" t="s">
+      <c r="M94" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="M94" s="6" t="s">
-        <v>159</v>
-      </c>
       <c r="N94" s="6" t="s">
         <v>27</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="P94" s="6" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
chore: atualiza CONTAS-A-RECEBER e remove arquivo temp do Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/CONTAS-A-RECEBER.xlsx
+++ b/planilhas/CONTAS-A-RECEBER.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -166,6 +166,9 @@
     <t>DAVI HENRIQUE DANTAS DE SOUZA</t>
   </si>
   <si>
+    <t>OLIZIEL DA SILVA CARDOSO</t>
+  </si>
+  <si>
     <t>FA-11562</t>
   </si>
   <si>
@@ -229,12 +232,6 @@
     <t>FA-11615</t>
   </si>
   <si>
-    <t>FA-11424</t>
-  </si>
-  <si>
-    <t>OLIZIEL DA SILVA CARDOSO</t>
-  </si>
-  <si>
     <t>FA-11489</t>
   </si>
   <si>
@@ -298,28 +295,31 @@
     <t>ND-11700</t>
   </si>
   <si>
+    <t>FA-11746</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11780</t>
+  </si>
+  <si>
     <t>FA-11718</t>
   </si>
   <si>
     <t>JOZILDO TARQUINO DE BRITO</t>
   </si>
   <si>
-    <t>FA-11746</t>
-  </si>
-  <si>
-    <t>ROBERTO MURATORI</t>
-  </si>
-  <si>
-    <t>FA-11780</t>
+    <t>FA-11566</t>
+  </si>
+  <si>
+    <t>DIEGO TAYAO DANTAS</t>
   </si>
   <si>
     <t>FA-11565</t>
   </si>
   <si>
-    <t>FA-11566</t>
-  </si>
-  <si>
-    <t>DIEGO TAYAO DANTAS</t>
+    <t>FA-11669</t>
   </si>
   <si>
     <t>FA-11721</t>
@@ -337,9 +337,6 @@
     <t>ANA FLORIPES CARVALHO DA CUNHA</t>
   </si>
   <si>
-    <t>FA-11669</t>
-  </si>
-  <si>
     <t>FA-11754</t>
   </si>
   <si>
@@ -373,24 +370,27 @@
     <t>DANILO DE ALMEIDA TORRES</t>
   </si>
   <si>
+    <t>FA-11657</t>
+  </si>
+  <si>
+    <t>LUCA ZOLI</t>
+  </si>
+  <si>
     <t>FA-11711</t>
   </si>
   <si>
     <t>FA-11774</t>
   </si>
   <si>
-    <t>FA-11657</t>
-  </si>
-  <si>
-    <t>LUCA ZOLI</t>
-  </si>
-  <si>
     <t>FA-11435</t>
   </si>
   <si>
     <t>RAYANE ROBERTA DA SILVA</t>
   </si>
   <si>
+    <t>FA-11413</t>
+  </si>
+  <si>
     <t>FA-11567</t>
   </si>
   <si>
@@ -400,18 +400,15 @@
     <t>FA-11677</t>
   </si>
   <si>
+    <t>FA-11772</t>
+  </si>
+  <si>
+    <t>FA-11760</t>
+  </si>
+  <si>
     <t>FA-11712</t>
   </si>
   <si>
-    <t>FA-11772</t>
-  </si>
-  <si>
-    <t>FA-11760</t>
-  </si>
-  <si>
-    <t>FA-11413</t>
-  </si>
-  <si>
     <t>FA-11778</t>
   </si>
   <si>
@@ -445,34 +442,34 @@
     <t>ELIONILSON CORDEIRO BARBOSA</t>
   </si>
   <si>
+    <t>FA-11579</t>
+  </si>
+  <si>
+    <t>ADRIANO TEOTONIO DA SILVA</t>
+  </si>
+  <si>
+    <t>LUZ DIVINA LTDA</t>
+  </si>
+  <si>
+    <t>FA-11592</t>
+  </si>
+  <si>
+    <t>JACKSON CASSIANO VERISSIMO</t>
+  </si>
+  <si>
+    <t>FA-11645</t>
+  </si>
+  <si>
+    <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
+  </si>
+  <si>
+    <t>PÚBLICO</t>
+  </si>
+  <si>
     <t>FA-11633</t>
   </si>
   <si>
     <t>TANIELLE GLAUCIANA SOUZA DA SILVA</t>
-  </si>
-  <si>
-    <t>PÚBLICO</t>
-  </si>
-  <si>
-    <t>LUZ DIVINA LTDA</t>
-  </si>
-  <si>
-    <t>FA-11579</t>
-  </si>
-  <si>
-    <t>ADRIANO TEOTONIO DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11592</t>
-  </si>
-  <si>
-    <t>JACKSON CASSIANO VERISSIMO</t>
-  </si>
-  <si>
-    <t>FA-11645</t>
-  </si>
-  <si>
-    <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
   </si>
 </sst>
 </file>
@@ -1672,8 +1669,8 @@
       <c r="D22" s="7">
         <v>46167</v>
       </c>
-      <c r="E22" s="7">
-        <v>46141</v>
+      <c r="E22" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F22" s="8">
         <v>-3</v>
@@ -1688,14 +1685,14 @@
         <v>30</v>
       </c>
       <c r="J22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L22" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K22" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L22" s="6" t="s">
-        <v>35</v>
-      </c>
       <c r="M22" s="6" t="s">
         <v>23</v>
       </c>
@@ -1709,13 +1706,13 @@
         <v>23</v>
       </c>
       <c r="Q22" s="6" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="R22" s="6" t="s">
         <v>37</v>
       </c>
       <c r="S22" s="9">
-        <v>310</v>
+        <v>249.21</v>
       </c>
     </row>
     <row r="23" ht="23" customHeight="1">
@@ -1726,16 +1723,16 @@
         <v>46167</v>
       </c>
       <c r="C23" s="7">
-        <v>46153</v>
+        <v>46167</v>
       </c>
       <c r="D23" s="7">
-        <v>46153</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>23</v>
+        <v>46167</v>
+      </c>
+      <c r="E23" s="7">
+        <v>46141</v>
       </c>
       <c r="F23" s="8">
-        <v>-17</v>
+        <v>-3</v>
       </c>
       <c r="G23" s="8">
         <v>-3</v>
@@ -1753,10 +1750,10 @@
         <v>23</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="N23" s="6" t="s">
         <v>27</v>
@@ -1768,13 +1765,13 @@
         <v>23</v>
       </c>
       <c r="Q23" s="6" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="R23" s="6" t="s">
         <v>37</v>
       </c>
       <c r="S23" s="9">
-        <v>400</v>
+        <v>310</v>
       </c>
     </row>
     <row r="24" ht="23" customHeight="1">
@@ -1785,16 +1782,16 @@
         <v>46167</v>
       </c>
       <c r="C24" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="D24" s="7">
-        <v>46160</v>
+        <v>46153</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F24" s="8">
-        <v>-10</v>
+        <v>-17</v>
       </c>
       <c r="G24" s="8">
         <v>-3</v>
@@ -1806,16 +1803,16 @@
         <v>30</v>
       </c>
       <c r="J24" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L24" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K24" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>48</v>
-      </c>
       <c r="M24" s="6" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="N24" s="6" t="s">
         <v>27</v>
@@ -1833,7 +1830,7 @@
         <v>37</v>
       </c>
       <c r="S24" s="9">
-        <v>572.72</v>
+        <v>400</v>
       </c>
     </row>
     <row r="25" ht="23" customHeight="1">
@@ -1844,16 +1841,16 @@
         <v>46167</v>
       </c>
       <c r="C25" s="7">
-        <v>46167</v>
+        <v>46160</v>
       </c>
       <c r="D25" s="7">
-        <v>46167</v>
+        <v>46160</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F25" s="8">
-        <v>-3</v>
+        <v>-10</v>
       </c>
       <c r="G25" s="8">
         <v>-3</v>
@@ -1865,14 +1862,14 @@
         <v>30</v>
       </c>
       <c r="J25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L25" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="K25" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="M25" s="6" t="s">
         <v>23</v>
       </c>
@@ -1889,10 +1886,10 @@
         <v>23</v>
       </c>
       <c r="R25" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="S25" s="9">
-        <v>600</v>
+        <v>572.72</v>
       </c>
     </row>
     <row r="26" ht="23" customHeight="1">
@@ -1908,8 +1905,8 @@
       <c r="D26" s="7">
         <v>46167</v>
       </c>
-      <c r="E26" s="7">
-        <v>46119</v>
+      <c r="E26" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="F26" s="8">
         <v>-3</v>
@@ -1924,16 +1921,16 @@
         <v>30</v>
       </c>
       <c r="J26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L26" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="K26" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L26" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="M26" s="6" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="N26" s="6" t="s">
         <v>27</v>
@@ -1945,10 +1942,10 @@
         <v>23</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S26" s="9">
         <v>600</v>
@@ -1968,7 +1965,7 @@
         <v>46167</v>
       </c>
       <c r="E27" s="7">
-        <v>46150</v>
+        <v>46119</v>
       </c>
       <c r="F27" s="8">
         <v>-3</v>
@@ -1989,10 +1986,10 @@
         <v>23</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="N27" s="6" t="s">
         <v>27</v>
@@ -2010,7 +2007,7 @@
         <v>37</v>
       </c>
       <c r="S27" s="9">
-        <v>630</v>
+        <v>600</v>
       </c>
     </row>
     <row r="28" ht="23" customHeight="1">
@@ -2027,7 +2024,7 @@
         <v>46167</v>
       </c>
       <c r="E28" s="7">
-        <v>46170</v>
+        <v>46150</v>
       </c>
       <c r="F28" s="8">
         <v>-3</v>
@@ -2042,16 +2039,16 @@
         <v>30</v>
       </c>
       <c r="J28" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L28" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="K28" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L28" s="6" t="s">
-        <v>46</v>
-      </c>
       <c r="M28" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="N28" s="6" t="s">
         <v>27</v>
@@ -2069,7 +2066,7 @@
         <v>37</v>
       </c>
       <c r="S28" s="9">
-        <v>650</v>
+        <v>630</v>
       </c>
     </row>
     <row r="29" ht="23" customHeight="1">
@@ -2086,7 +2083,7 @@
         <v>46167</v>
       </c>
       <c r="E29" s="7">
-        <v>46113</v>
+        <v>46170</v>
       </c>
       <c r="F29" s="8">
         <v>-3</v>
@@ -2107,10 +2104,10 @@
         <v>23</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N29" s="6" t="s">
         <v>27</v>
@@ -2128,7 +2125,7 @@
         <v>37</v>
       </c>
       <c r="S29" s="9">
-        <v>680</v>
+        <v>650</v>
       </c>
     </row>
     <row r="30" ht="23" customHeight="1">
@@ -2145,7 +2142,7 @@
         <v>46167</v>
       </c>
       <c r="E30" s="7">
-        <v>46164</v>
+        <v>46113</v>
       </c>
       <c r="F30" s="8">
         <v>-3</v>
@@ -2166,10 +2163,10 @@
         <v>23</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="N30" s="6" t="s">
         <v>27</v>
@@ -2184,7 +2181,7 @@
         <v>36</v>
       </c>
       <c r="R30" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="S30" s="9">
         <v>680</v>
@@ -2204,7 +2201,7 @@
         <v>46167</v>
       </c>
       <c r="E31" s="7">
-        <v>46168</v>
+        <v>46164</v>
       </c>
       <c r="F31" s="8">
         <v>-3</v>
@@ -2219,13 +2216,13 @@
         <v>30</v>
       </c>
       <c r="J31" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="K31" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L31" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="M31" s="6" t="s">
         <v>23</v>
@@ -2243,7 +2240,7 @@
         <v>36</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S31" s="9">
         <v>680</v>
@@ -2263,7 +2260,7 @@
         <v>46167</v>
       </c>
       <c r="E32" s="7">
-        <v>46141</v>
+        <v>46168</v>
       </c>
       <c r="F32" s="8">
         <v>-3</v>
@@ -2278,13 +2275,13 @@
         <v>30</v>
       </c>
       <c r="J32" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L32" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="K32" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>23</v>
@@ -2302,7 +2299,7 @@
         <v>36</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="S32" s="9">
         <v>680</v>
@@ -2322,7 +2319,7 @@
         <v>46167</v>
       </c>
       <c r="E33" s="7">
-        <v>46167</v>
+        <v>46141</v>
       </c>
       <c r="F33" s="8">
         <v>-3</v>
@@ -2337,13 +2334,13 @@
         <v>30</v>
       </c>
       <c r="J33" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="K33" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>63</v>
       </c>
       <c r="M33" s="6" t="s">
         <v>23</v>
@@ -2361,7 +2358,7 @@
         <v>36</v>
       </c>
       <c r="R33" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S33" s="9">
         <v>680</v>
@@ -2372,22 +2369,22 @@
         <v>22</v>
       </c>
       <c r="B34" s="7">
-        <v>46168</v>
+        <v>46167</v>
       </c>
       <c r="C34" s="7">
-        <v>46153</v>
+        <v>46167</v>
       </c>
       <c r="D34" s="7">
-        <v>46153</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>23</v>
+        <v>46167</v>
+      </c>
+      <c r="E34" s="7">
+        <v>46167</v>
       </c>
       <c r="F34" s="8">
-        <v>-17</v>
+        <v>-3</v>
       </c>
       <c r="G34" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>30</v>
@@ -2396,14 +2393,14 @@
         <v>30</v>
       </c>
       <c r="J34" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L34" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="M34" s="6" t="s">
         <v>23</v>
       </c>
@@ -2417,13 +2414,13 @@
         <v>23</v>
       </c>
       <c r="Q34" s="6" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="R34" s="6" t="s">
         <v>37</v>
       </c>
       <c r="S34" s="9">
-        <v>13.43</v>
+        <v>680</v>
       </c>
     </row>
     <row r="35" ht="23" customHeight="1">
@@ -2434,22 +2431,22 @@
         <v>46168</v>
       </c>
       <c r="C35" s="7">
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="D35" s="7">
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>23</v>
       </c>
       <c r="F35" s="8">
-        <v>-38</v>
+        <v>-17</v>
       </c>
       <c r="G35" s="8">
         <v>-2</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>30</v>
@@ -2461,7 +2458,7 @@
         <v>23</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>23</v>
@@ -2482,7 +2479,7 @@
         <v>37</v>
       </c>
       <c r="S35" s="9">
-        <v>249.21</v>
+        <v>13.43</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1">
@@ -2514,13 +2511,13 @@
         <v>30</v>
       </c>
       <c r="J36" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L36" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>23</v>
@@ -2573,13 +2570,13 @@
         <v>30</v>
       </c>
       <c r="J37" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L37" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="K37" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>23</v>
@@ -2632,13 +2629,13 @@
         <v>30</v>
       </c>
       <c r="J38" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L38" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="K38" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L38" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>23</v>
@@ -2691,16 +2688,16 @@
         <v>30</v>
       </c>
       <c r="J39" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L39" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="K39" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="M39" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N39" s="6" t="s">
         <v>27</v>
@@ -2750,22 +2747,22 @@
         <v>23</v>
       </c>
       <c r="J40" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M40" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O40" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="K40" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L40" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="M40" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="N40" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O40" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>23</v>
@@ -2809,25 +2806,25 @@
         <v>23</v>
       </c>
       <c r="J41" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L41" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="K41" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L41" s="6" t="s">
+      <c r="M41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N41" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O41" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="P41" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="M41" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N41" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O41" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="P41" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="Q41" s="6" t="s">
         <v>23</v>
@@ -2868,13 +2865,13 @@
         <v>23</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K42" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M42" s="6" t="s">
         <v>23</v>
@@ -2883,7 +2880,7 @@
         <v>27</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>23</v>
@@ -2927,14 +2924,14 @@
         <v>23</v>
       </c>
       <c r="J43" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L43" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="K43" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L43" s="6" t="s">
-        <v>82</v>
-      </c>
       <c r="M43" s="6" t="s">
         <v>23</v>
       </c>
@@ -2942,7 +2939,7 @@
         <v>27</v>
       </c>
       <c r="O43" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P43" s="6" t="s">
         <v>23</v>
@@ -2992,16 +2989,16 @@
         <v>23</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M44" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>23</v>
@@ -3045,25 +3042,25 @@
         <v>23</v>
       </c>
       <c r="J45" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L45" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="K45" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L45" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="M45" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O45" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P45" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q45" s="6" t="s">
         <v>29</v>
@@ -3104,22 +3101,22 @@
         <v>23</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="M46" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>23</v>
@@ -3175,10 +3172,10 @@
         <v>23</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O47" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P47" s="6" t="s">
         <v>23</v>
@@ -3222,22 +3219,22 @@
         <v>23</v>
       </c>
       <c r="J48" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L48" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="K48" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L48" s="6" t="s">
-        <v>89</v>
-      </c>
       <c r="M48" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>23</v>
@@ -3266,7 +3263,7 @@
         <v>46174</v>
       </c>
       <c r="E49" s="7">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="F49" s="8">
         <v>4</v>
@@ -3281,22 +3278,22 @@
         <v>23</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K49" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P49" s="6" t="s">
         <v>23</v>
@@ -3325,7 +3322,7 @@
         <v>46174</v>
       </c>
       <c r="E50" s="7">
-        <v>46170</v>
+        <v>46169</v>
       </c>
       <c r="F50" s="8">
         <v>4</v>
@@ -3340,22 +3337,22 @@
         <v>23</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="K50" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>23</v>
@@ -3399,22 +3396,22 @@
         <v>23</v>
       </c>
       <c r="J51" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L51" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="K51" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>35</v>
-      </c>
       <c r="M51" s="6" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O51" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P51" s="6" t="s">
         <v>23</v>
@@ -3464,16 +3461,16 @@
         <v>23</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>95</v>
+        <v>23</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>23</v>
@@ -3502,7 +3499,7 @@
         <v>46174</v>
       </c>
       <c r="E53" s="7">
-        <v>46169</v>
+        <v>46163</v>
       </c>
       <c r="F53" s="8">
         <v>4</v>
@@ -3517,22 +3514,22 @@
         <v>23</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K53" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="M53" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O53" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P53" s="6" t="s">
         <v>23</v>
@@ -3576,22 +3573,22 @@
         <v>23</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="K54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>23</v>
@@ -3635,22 +3632,22 @@
         <v>23</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K55" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="M55" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P55" s="6" t="s">
         <v>23</v>
@@ -3679,7 +3676,7 @@
         <v>46174</v>
       </c>
       <c r="E56" s="7">
-        <v>46163</v>
+        <v>46169</v>
       </c>
       <c r="F56" s="8">
         <v>4</v>
@@ -3694,22 +3691,22 @@
         <v>23</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>23</v>
@@ -3753,22 +3750,22 @@
         <v>23</v>
       </c>
       <c r="J57" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L57" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="K57" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L57" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="M57" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O57" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P57" s="6" t="s">
         <v>23</v>
@@ -3812,25 +3809,25 @@
         <v>23</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K58" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M58" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>36</v>
@@ -3871,22 +3868,22 @@
         <v>23</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K59" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M59" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O59" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P59" s="6" t="s">
         <v>23</v>
@@ -3930,22 +3927,22 @@
         <v>23</v>
       </c>
       <c r="J60" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="K60" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L60" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="K60" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L60" s="6" t="s">
-        <v>107</v>
-      </c>
       <c r="M60" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>23</v>
@@ -3989,22 +3986,22 @@
         <v>23</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K61" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M61" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O61" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P61" s="6" t="s">
         <v>23</v>
@@ -4048,22 +4045,22 @@
         <v>23</v>
       </c>
       <c r="J62" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="K62" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L62" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="K62" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L62" s="6" t="s">
-        <v>110</v>
-      </c>
       <c r="M62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>23</v>
@@ -4107,22 +4104,22 @@
         <v>23</v>
       </c>
       <c r="J63" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L63" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="K63" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L63" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="M63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O63" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P63" s="6" t="s">
         <v>23</v>
@@ -4151,7 +4148,7 @@
         <v>46174</v>
       </c>
       <c r="E64" s="7">
-        <v>46168</v>
+        <v>46160</v>
       </c>
       <c r="F64" s="8">
         <v>4</v>
@@ -4166,22 +4163,22 @@
         <v>23</v>
       </c>
       <c r="J64" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L64" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="K64" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L64" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="M64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>23</v>
@@ -4190,7 +4187,7 @@
         <v>36</v>
       </c>
       <c r="R64" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="S64" s="9">
         <v>650</v>
@@ -4210,7 +4207,7 @@
         <v>46174</v>
       </c>
       <c r="E65" s="7">
-        <v>46170</v>
+        <v>46168</v>
       </c>
       <c r="F65" s="8">
         <v>4</v>
@@ -4231,16 +4228,16 @@
         <v>23</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O65" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P65" s="6" t="s">
         <v>23</v>
@@ -4249,7 +4246,7 @@
         <v>36</v>
       </c>
       <c r="R65" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S65" s="9">
         <v>650</v>
@@ -4269,7 +4266,7 @@
         <v>46174</v>
       </c>
       <c r="E66" s="7">
-        <v>46160</v>
+        <v>46170</v>
       </c>
       <c r="F66" s="8">
         <v>4</v>
@@ -4290,16 +4287,16 @@
         <v>23</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="M66" s="6" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>23</v>
@@ -4343,22 +4340,22 @@
         <v>23</v>
       </c>
       <c r="J67" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L67" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="K67" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L67" s="6" t="s">
-        <v>118</v>
-      </c>
       <c r="M67" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P67" s="6" t="s">
         <v>23</v>
@@ -4387,7 +4384,7 @@
         <v>46174</v>
       </c>
       <c r="E68" s="7">
-        <v>46141</v>
+        <v>46113</v>
       </c>
       <c r="F68" s="8">
         <v>4</v>
@@ -4402,22 +4399,22 @@
         <v>23</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K68" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="M68" s="6" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>23</v>
@@ -4426,7 +4423,7 @@
         <v>36</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="S68" s="9">
         <v>680</v>
@@ -4446,7 +4443,7 @@
         <v>46174</v>
       </c>
       <c r="E69" s="7">
-        <v>46167</v>
+        <v>46141</v>
       </c>
       <c r="F69" s="8">
         <v>4</v>
@@ -4461,22 +4458,22 @@
         <v>23</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K69" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O69" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P69" s="6" t="s">
         <v>23</v>
@@ -4485,7 +4482,7 @@
         <v>36</v>
       </c>
       <c r="R69" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S69" s="9">
         <v>680</v>
@@ -4505,7 +4502,7 @@
         <v>46174</v>
       </c>
       <c r="E70" s="7">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="F70" s="8">
         <v>4</v>
@@ -4520,22 +4517,22 @@
         <v>23</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K70" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="M70" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>23</v>
@@ -4544,7 +4541,7 @@
         <v>36</v>
       </c>
       <c r="R70" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="S70" s="9">
         <v>680</v>
@@ -4564,7 +4561,7 @@
         <v>46174</v>
       </c>
       <c r="E71" s="7">
-        <v>46168</v>
+        <v>46164</v>
       </c>
       <c r="F71" s="8">
         <v>4</v>
@@ -4579,22 +4576,22 @@
         <v>23</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K71" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M71" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O71" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P71" s="6" t="s">
         <v>23</v>
@@ -4603,7 +4600,7 @@
         <v>36</v>
       </c>
       <c r="R71" s="6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S71" s="9">
         <v>680</v>
@@ -4638,22 +4635,22 @@
         <v>23</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="M72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>23</v>
@@ -4697,22 +4694,22 @@
         <v>23</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O73" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P73" s="6" t="s">
         <v>23</v>
@@ -4741,7 +4738,7 @@
         <v>46174</v>
       </c>
       <c r="E74" s="7">
-        <v>46113</v>
+        <v>46168</v>
       </c>
       <c r="F74" s="8">
         <v>4</v>
@@ -4756,22 +4753,22 @@
         <v>23</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K74" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="M74" s="6" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>23</v>
@@ -4815,25 +4812,25 @@
         <v>23</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K75" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L75" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="M75" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N75" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="O75" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="P75" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="M75" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N75" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="O75" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="P75" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="Q75" s="6" t="s">
         <v>36</v>
@@ -4874,22 +4871,22 @@
         <v>23</v>
       </c>
       <c r="J76" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L76" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K76" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L76" s="6" t="s">
-        <v>128</v>
-      </c>
       <c r="M76" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>23</v>
@@ -4933,22 +4930,22 @@
         <v>23</v>
       </c>
       <c r="J77" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K77" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L77" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="K77" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L77" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="M77" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O77" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P77" s="6" t="s">
         <v>23</v>
@@ -4992,22 +4989,22 @@
         <v>23</v>
       </c>
       <c r="J78" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L78" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="K78" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L78" s="6" t="s">
-        <v>132</v>
-      </c>
       <c r="M78" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>23</v>
@@ -5016,7 +5013,7 @@
         <v>36</v>
       </c>
       <c r="R78" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="S78" s="9">
         <v>800</v>
@@ -5024,7 +5021,7 @@
     </row>
     <row r="79" ht="23" customHeight="1">
       <c r="A79" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B79" s="7">
         <v>46174</v>
@@ -5051,22 +5048,22 @@
         <v>23</v>
       </c>
       <c r="J79" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L79" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="K79" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L79" s="6" t="s">
-        <v>136</v>
-      </c>
       <c r="M79" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N79" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O79" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P79" s="6" t="s">
         <v>23</v>
@@ -5075,7 +5072,7 @@
         <v>36</v>
       </c>
       <c r="R79" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="S79" s="9">
         <v>800</v>
@@ -5095,7 +5092,7 @@
         <v>46174</v>
       </c>
       <c r="E80" s="7">
-        <v>46160</v>
+        <v>46148</v>
       </c>
       <c r="F80" s="8">
         <v>4</v>
@@ -5110,31 +5107,31 @@
         <v>23</v>
       </c>
       <c r="J80" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L80" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="K80" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L80" s="6" t="s">
-        <v>138</v>
-      </c>
       <c r="M80" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>139</v>
+        <v>23</v>
       </c>
       <c r="Q80" s="6" t="s">
         <v>36</v>
       </c>
       <c r="R80" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="S80" s="9">
         <v>1200</v>
@@ -5169,22 +5166,22 @@
         <v>23</v>
       </c>
       <c r="J81" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="K81" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="M81" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N81" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O81" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P81" s="6" t="s">
         <v>23</v>
@@ -5193,7 +5190,7 @@
         <v>36</v>
       </c>
       <c r="R81" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="S81" s="9">
         <v>1200</v>
@@ -5213,7 +5210,7 @@
         <v>46174</v>
       </c>
       <c r="E82" s="7">
-        <v>46148</v>
+        <v>46160</v>
       </c>
       <c r="F82" s="8">
         <v>4</v>
@@ -5228,31 +5225,31 @@
         <v>23</v>
       </c>
       <c r="J82" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N82" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="O82" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="P82" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="K82" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L82" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="M82" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N82" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="O82" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="P82" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="Q82" s="6" t="s">
         <v>36</v>
       </c>
       <c r="R82" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="S82" s="9">
         <v>1200</v>
@@ -5287,31 +5284,31 @@
         <v>23</v>
       </c>
       <c r="J83" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="K83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L83" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="K83" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L83" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="M83" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N83" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O83" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P83" s="6" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="Q83" s="6" t="s">
         <v>36</v>
       </c>
       <c r="R83" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="S83" s="9">
         <v>1200</v>

</xml_diff>